<commit_message>
feat: Add presentation HTML, ppt script, and slide 5 typewriter effect
</commit_message>
<xml_diff>
--- a/작업장소 (영수증 보관)/2026-06/심천지사 전도금 정산 양식_2026-06.xlsx
+++ b/작업장소 (영수증 보관)/2026-06/심천지사 전도금 정산 양식_2026-06.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="603" firstSheet="0" activeTab="6" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="603" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="통장내역(환율표)" sheetId="1" state="visible" r:id="rId1"/>
@@ -5132,6 +5132,27 @@
     <xf numFmtId="168" fontId="76" fillId="2" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="168" fontId="76" fillId="2" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="76" fillId="2" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="137">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="77" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="138">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="71" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="138">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="15" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="2">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5209,27 +5230,6 @@
     </xf>
     <xf numFmtId="0" fontId="67" fillId="2" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="176">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="76" fillId="2" borderId="43" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="76" fillId="2" borderId="44" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="71" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="137">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="77" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="138">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="170" fontId="71" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="138">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="15" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="20" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="563">
@@ -7390,293 +7390,6 @@
 </comments>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>38</row>
-      <rowOff>158750</rowOff>
-    </from>
-    <to>
-      <col>10</col>
-      <colOff>603249</colOff>
-      <row>83</row>
-      <rowOff>36703</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="图片 14"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="0" y="6953250"/>
-          <a:ext cx="9405937" cy="7736078"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>142876</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>9</col>
-      <colOff>127000</colOff>
-      <row>36</row>
-      <rowOff>165491</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="图片 13"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="142876" y="0"/>
-          <a:ext cx="8159749" cy="6586929"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>8</col>
-      <colOff>619124</colOff>
-      <row>0</row>
-      <rowOff>119063</rowOff>
-    </from>
-    <to>
-      <col>20</col>
-      <colOff>395384</colOff>
-      <row>33</row>
-      <rowOff>111125</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="图片 12"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="8167687" y="119063"/>
-          <a:ext cx="7324822" cy="5889625"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>83</row>
-      <rowOff>31750</rowOff>
-    </from>
-    <to>
-      <col>10</col>
-      <colOff>476250</colOff>
-      <row>97</row>
-      <rowOff>105569</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="图片 15"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="0" y="14684375"/>
-          <a:ext cx="9278938" cy="2518569"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>97</row>
-      <rowOff>87313</rowOff>
-    </from>
-    <to>
-      <col>10</col>
-      <colOff>484186</colOff>
-      <row>112</row>
-      <rowOff>2441</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="图片 16"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId6"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="0" y="17184688"/>
-          <a:ext cx="9286874" cy="2534503"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>111</row>
-      <rowOff>75406</rowOff>
-    </from>
-    <to>
-      <col>10</col>
-      <colOff>508000</colOff>
-      <row>120</row>
-      <rowOff>69712</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="22" name="图片 21"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId7"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="0" y="23911719"/>
-          <a:ext cx="10175875" cy="1923118"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>12</col>
-      <colOff>371515</colOff>
-      <row>66</row>
-      <rowOff>3669</rowOff>
-    </from>
-    <ext cx="7263148" cy="8509715"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="그림 3"/>
-        <cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm>
-          <a:off x="8601115" y="13833969"/>
-          <a:ext cx="7263148" cy="8509715"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <avLst/>
-        </a:prstGeom>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
 <externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <externalBook r:id="rId1">
@@ -8220,36 +7933,36 @@
           <t>지급</t>
         </is>
       </c>
-      <c r="D2" s="624" t="n"/>
-      <c r="E2" s="620" t="n"/>
+      <c r="D2" s="631" t="n"/>
+      <c r="E2" s="627" t="n"/>
       <c r="F2" s="656" t="inlineStr">
         <is>
           <t>송금액</t>
         </is>
       </c>
-      <c r="G2" s="624" t="n"/>
-      <c r="H2" s="620" t="n"/>
+      <c r="G2" s="631" t="n"/>
+      <c r="H2" s="627" t="n"/>
       <c r="I2" s="656" t="inlineStr">
         <is>
           <t>입금</t>
         </is>
       </c>
-      <c r="J2" s="620" t="n"/>
+      <c r="J2" s="627" t="n"/>
       <c r="K2" s="656" t="inlineStr">
         <is>
           <t>출금</t>
         </is>
       </c>
-      <c r="L2" s="620" t="n"/>
-      <c r="M2" s="619" t="inlineStr">
+      <c r="L2" s="627" t="n"/>
+      <c r="M2" s="626" t="inlineStr">
         <is>
           <t>잔액</t>
         </is>
       </c>
-      <c r="N2" s="620" t="n"/>
+      <c r="N2" s="627" t="n"/>
     </row>
     <row r="3" ht="27" customHeight="1" s="654">
-      <c r="B3" s="622" t="n"/>
+      <c r="B3" s="629" t="n"/>
       <c r="C3" s="657" t="inlineStr">
         <is>
           <t>지급시
@@ -10688,43 +10401,33 @@
           <t>심천지사</t>
         </is>
       </c>
-      <c r="F5" s="409" t="n">
-        <v>6</v>
-      </c>
+      <c r="F5" s="409" t="n"/>
       <c r="G5" s="409">
         <f>F5*20</f>
         <v/>
       </c>
       <c r="H5" s="409" t="n"/>
-      <c r="J5" s="1123" t="n">
-        <v>46135</v>
-      </c>
+      <c r="J5" s="1123" t="n"/>
       <c r="K5" s="409" t="n"/>
       <c r="L5" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="M5" s="409" t="n">
-        <v>4</v>
-      </c>
+      <c r="M5" s="409" t="n"/>
       <c r="N5" s="409">
         <f>M5*20</f>
         <v/>
       </c>
       <c r="O5" s="409" t="n"/>
-      <c r="Q5" s="1123" t="n">
-        <v>46134</v>
-      </c>
+      <c r="Q5" s="1123" t="n"/>
       <c r="R5" s="409" t="n"/>
       <c r="S5" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="T5" s="409" t="n">
-        <v>1</v>
-      </c>
+      <c r="T5" s="409" t="n"/>
       <c r="U5" s="409">
         <f>T5*20</f>
         <v/>
@@ -10732,52 +10435,40 @@
       <c r="V5" s="409" t="n"/>
     </row>
     <row r="6">
-      <c r="C6" s="1123" t="n">
-        <v>46135</v>
-      </c>
+      <c r="C6" s="1123" t="n"/>
       <c r="D6" s="409" t="n"/>
       <c r="E6" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="F6" s="409" t="n">
-        <v>3.5</v>
-      </c>
+      <c r="F6" s="409" t="n"/>
       <c r="G6" s="409">
         <f>F6*20</f>
         <v/>
       </c>
       <c r="H6" s="409" t="n"/>
-      <c r="J6" s="1123" t="n">
-        <v>46139</v>
-      </c>
+      <c r="J6" s="1123" t="n"/>
       <c r="K6" s="409" t="n"/>
       <c r="L6" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="M6" s="409" t="n">
-        <v>4</v>
-      </c>
+      <c r="M6" s="409" t="n"/>
       <c r="N6" s="409">
         <f>M6*20</f>
         <v/>
       </c>
       <c r="O6" s="409" t="n"/>
-      <c r="Q6" s="1123" t="n">
-        <v>46135</v>
-      </c>
+      <c r="Q6" s="1123" t="n"/>
       <c r="R6" s="409" t="n"/>
       <c r="S6" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="T6" s="409" t="n">
-        <v>2</v>
-      </c>
+      <c r="T6" s="409" t="n"/>
       <c r="U6" s="409">
         <f>T6*20</f>
         <v/>
@@ -10785,52 +10476,40 @@
       <c r="V6" s="409" t="n"/>
     </row>
     <row r="7">
-      <c r="C7" s="1123" t="n">
-        <v>46136</v>
-      </c>
+      <c r="C7" s="1123" t="n"/>
       <c r="D7" s="409" t="n"/>
       <c r="E7" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="F7" s="409" t="n">
-        <v>6.5</v>
-      </c>
+      <c r="F7" s="409" t="n"/>
       <c r="G7" s="409">
         <f>F7*20</f>
         <v/>
       </c>
       <c r="H7" s="409" t="n"/>
-      <c r="J7" s="1123" t="n">
-        <v>46149</v>
-      </c>
+      <c r="J7" s="1123" t="n"/>
       <c r="K7" s="409" t="n"/>
       <c r="L7" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="M7" s="409" t="n">
-        <v>3</v>
-      </c>
+      <c r="M7" s="409" t="n"/>
       <c r="N7" s="409">
         <f>M7*20</f>
         <v/>
       </c>
       <c r="O7" s="409" t="n"/>
-      <c r="Q7" s="1123" t="n">
-        <v>46139</v>
-      </c>
+      <c r="Q7" s="1123" t="n"/>
       <c r="R7" s="409" t="n"/>
       <c r="S7" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="T7" s="409" t="n">
-        <v>3</v>
-      </c>
+      <c r="T7" s="409" t="n"/>
       <c r="U7" s="409">
         <f>T7*20</f>
         <v/>
@@ -10838,52 +10517,40 @@
       <c r="V7" s="409" t="n"/>
     </row>
     <row r="8">
-      <c r="C8" s="1123" t="n">
-        <v>46139</v>
-      </c>
+      <c r="C8" s="1123" t="n"/>
       <c r="D8" s="409" t="n"/>
       <c r="E8" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="F8" s="409" t="n">
-        <v>3</v>
-      </c>
+      <c r="F8" s="409" t="n"/>
       <c r="G8" s="409">
         <f>F8*20</f>
         <v/>
       </c>
       <c r="H8" s="409" t="n"/>
-      <c r="J8" s="1123" t="n">
-        <v>46150</v>
-      </c>
+      <c r="J8" s="1123" t="n"/>
       <c r="K8" s="409" t="n"/>
       <c r="L8" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="M8" s="409" t="n">
-        <v>3</v>
-      </c>
+      <c r="M8" s="409" t="n"/>
       <c r="N8" s="409">
         <f>M8*20</f>
         <v/>
       </c>
       <c r="O8" s="409" t="n"/>
-      <c r="Q8" s="1123" t="n">
-        <v>46140</v>
-      </c>
+      <c r="Q8" s="1123" t="n"/>
       <c r="R8" s="409" t="n"/>
       <c r="S8" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="T8" s="409" t="n">
-        <v>1</v>
-      </c>
+      <c r="T8" s="409" t="n"/>
       <c r="U8" s="409">
         <f>T8*20</f>
         <v/>
@@ -10891,52 +10558,40 @@
       <c r="V8" s="409" t="n"/>
     </row>
     <row r="9">
-      <c r="C9" s="1123" t="n">
-        <v>46142</v>
-      </c>
+      <c r="C9" s="1123" t="n"/>
       <c r="D9" s="409" t="n"/>
       <c r="E9" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="F9" s="409" t="n">
-        <v>1</v>
-      </c>
+      <c r="F9" s="409" t="n"/>
       <c r="G9" s="409">
         <f>F9*20</f>
         <v/>
       </c>
       <c r="H9" s="411" t="n"/>
-      <c r="J9" s="1123" t="n">
-        <v>46155</v>
-      </c>
+      <c r="J9" s="1123" t="n"/>
       <c r="K9" s="409" t="n"/>
       <c r="L9" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="M9" s="409" t="n">
-        <v>5</v>
-      </c>
+      <c r="M9" s="409" t="n"/>
       <c r="N9" s="409">
         <f>M9*20</f>
         <v/>
       </c>
       <c r="O9" s="411" t="n"/>
-      <c r="Q9" s="1123" t="n">
-        <v>46154</v>
-      </c>
+      <c r="Q9" s="1123" t="n"/>
       <c r="R9" s="409" t="n"/>
       <c r="S9" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="T9" s="409" t="n">
-        <v>3</v>
-      </c>
+      <c r="T9" s="409" t="n"/>
       <c r="U9" s="409">
         <f>T9*20</f>
         <v/>
@@ -10944,52 +10599,40 @@
       <c r="V9" s="411" t="n"/>
     </row>
     <row r="10">
-      <c r="C10" s="1123" t="n">
-        <v>46150</v>
-      </c>
+      <c r="C10" s="1123" t="n"/>
       <c r="D10" s="409" t="n"/>
       <c r="E10" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="F10" s="409" t="n">
-        <v>5</v>
-      </c>
+      <c r="F10" s="409" t="n"/>
       <c r="G10" s="409">
         <f>F10*20</f>
         <v/>
       </c>
       <c r="H10" s="409" t="n"/>
-      <c r="J10" s="1123" t="n">
-        <v>46158</v>
-      </c>
+      <c r="J10" s="1123" t="n"/>
       <c r="K10" s="409" t="n"/>
       <c r="L10" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="M10" s="409" t="n">
-        <v>16</v>
-      </c>
+      <c r="M10" s="409" t="n"/>
       <c r="N10" s="409">
         <f>M10*20</f>
         <v/>
       </c>
       <c r="O10" s="409" t="n"/>
-      <c r="Q10" s="1123" t="n">
-        <v>46158</v>
-      </c>
+      <c r="Q10" s="1123" t="n"/>
       <c r="R10" s="409" t="n"/>
       <c r="S10" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="T10" s="409" t="n">
-        <v>5</v>
-      </c>
+      <c r="T10" s="409" t="n"/>
       <c r="U10" s="409">
         <f>T10*20</f>
         <v/>
@@ -10997,35 +10640,27 @@
       <c r="V10" s="409" t="n"/>
     </row>
     <row r="11">
-      <c r="C11" s="1123" t="n">
-        <v>46153</v>
-      </c>
+      <c r="C11" s="1123" t="n"/>
       <c r="D11" s="409" t="n"/>
       <c r="E11" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="F11" s="409" t="n">
-        <v>1</v>
-      </c>
+      <c r="F11" s="409" t="n"/>
       <c r="G11" s="409">
         <f>F11*20</f>
         <v/>
       </c>
       <c r="H11" s="409" t="n"/>
-      <c r="J11" s="1123" t="n">
-        <v>46159</v>
-      </c>
+      <c r="J11" s="1123" t="n"/>
       <c r="K11" s="409" t="n"/>
       <c r="L11" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="M11" s="409" t="n">
-        <v>3</v>
-      </c>
+      <c r="M11" s="409" t="n"/>
       <c r="N11" s="409">
         <f>M11*20</f>
         <v/>
@@ -11046,18 +10681,14 @@
       <c r="V11" s="409" t="n"/>
     </row>
     <row r="12">
-      <c r="C12" s="1123" t="n">
-        <v>46156</v>
-      </c>
+      <c r="C12" s="1123" t="n"/>
       <c r="D12" s="409" t="n"/>
       <c r="E12" s="409" t="inlineStr">
         <is>
           <t>심천지사</t>
         </is>
       </c>
-      <c r="F12" s="409" t="n">
-        <v>3</v>
-      </c>
+      <c r="F12" s="409" t="n"/>
       <c r="G12" s="409">
         <f>F12*20</f>
         <v/>
@@ -41705,7 +41336,7 @@
         </is>
       </c>
       <c r="Q79" s="971" t="n"/>
-      <c r="R79" s="637" t="inlineStr">
+      <c r="R79" s="644" t="inlineStr">
         <is>
           <t>김명관
 수석</t>
@@ -42030,7 +41661,7 @@
         </is>
       </c>
       <c r="Q84" s="971" t="n"/>
-      <c r="R84" s="637" t="inlineStr">
+      <c r="R84" s="644" t="inlineStr">
         <is>
           <t>신순연
 책임</t>
@@ -42355,7 +41986,7 @@
         </is>
       </c>
       <c r="Q89" s="971" t="n"/>
-      <c r="R89" s="637" t="inlineStr">
+      <c r="R89" s="644" t="inlineStr">
         <is>
           <t>FAE (Pan Shi Qiang)
 7/1 입사
@@ -42637,7 +42268,7 @@
         </is>
       </c>
       <c r="Q94" s="971" t="n"/>
-      <c r="R94" s="639" t="inlineStr">
+      <c r="R94" s="646" t="inlineStr">
         <is>
           <t>张亮(Zhang Liang)
 23/8/1 입사</t>
@@ -42908,7 +42539,7 @@
         </is>
       </c>
       <c r="Q99" s="971" t="n"/>
-      <c r="R99" s="637" t="inlineStr">
+      <c r="R99" s="644" t="inlineStr">
         <is>
           <t>林洁婷 임결정
 23/9/18 입사</t>
@@ -43126,7 +42757,7 @@
         </is>
       </c>
       <c r="Q103" s="971" t="n"/>
-      <c r="R103" s="637" t="inlineStr">
+      <c r="R103" s="644" t="inlineStr">
         <is>
           <t>朴美玲 박미령
 23/9/18 입사</t>
@@ -43598,14 +43229,14 @@
   <mergeCells count="11">
     <mergeCell ref="N17:O17"/>
     <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="R94:R98"/>
     <mergeCell ref="P17:Q17"/>
     <mergeCell ref="R79:R83"/>
+    <mergeCell ref="R103:R107"/>
     <mergeCell ref="R84:R88"/>
     <mergeCell ref="R89:R93"/>
     <mergeCell ref="K17:M17"/>
     <mergeCell ref="H17:J17"/>
-    <mergeCell ref="R103:R107"/>
+    <mergeCell ref="R94:R98"/>
     <mergeCell ref="R99:R102"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -43665,7 +43296,7 @@
       <c r="P1" s="999" t="n"/>
       <c r="Q1" s="999" t="n"/>
       <c r="R1" s="1000" t="n"/>
-      <c r="S1" s="649" t="n"/>
+      <c r="S1" s="621" t="n"/>
     </row>
     <row r="2" ht="15" customHeight="1" s="654">
       <c r="B2" s="1001" t="inlineStr">
@@ -44495,7 +44126,11 @@
     </row>
     <row r="21" ht="11.1" customFormat="1" customHeight="1" s="1089">
       <c r="A21" s="537" t="n"/>
-      <c r="B21" s="1090" t="n"/>
+      <c r="B21" s="1090" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
       <c r="C21" s="1090" t="n"/>
       <c r="D21" s="1090" t="n"/>
       <c r="E21" s="608" t="n"/>
@@ -44509,9 +44144,11 @@
       <c r="M21" s="1091" t="n"/>
       <c r="N21" s="1092" t="n"/>
       <c r="O21" s="1093" t="n"/>
-      <c r="P21" s="1094" t="n"/>
+      <c r="P21" s="1094" t="n">
+        <v>-315167.5839999999</v>
+      </c>
       <c r="Q21" s="1094" t="n">
-        <v>0</v>
+        <v>-47280.84835484935</v>
       </c>
       <c r="R21" s="1095" t="n"/>
       <c r="S21" s="1096" t="n"/>
@@ -44567,10 +44204,7 @@
         <v>74959.75</v>
       </c>
       <c r="M22" s="1099" t="n"/>
-      <c r="N22" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
-        <v/>
-      </c>
+      <c r="N22" s="1100" t="n"/>
       <c r="O22" s="1101" t="inlineStr"/>
       <c r="P22" s="1102">
         <f>P21+J22-M22</f>
@@ -44632,11 +44266,11 @@
       <c r="J23" s="601" t="n"/>
       <c r="K23" s="601" t="n"/>
       <c r="L23" s="601" t="n"/>
-      <c r="M23" s="1099" t="n"/>
-      <c r="N23" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
-        <v/>
-      </c>
+      <c r="M23" s="1099">
+        <f>O23*N23</f>
+        <v/>
+      </c>
+      <c r="N23" s="1100" t="n"/>
       <c r="O23" s="1101" t="n">
         <v>25</v>
       </c>
@@ -44689,12 +44323,12 @@
       </c>
       <c r="H24" s="600" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I24" s="599" t="inlineStr">
         <is>
-          <t>전도금 입금</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J24" s="601" t="n"/>
@@ -44704,7 +44338,7 @@
         <v>44</v>
       </c>
       <c r="N24" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O24" s="1101">
@@ -44759,22 +44393,22 @@
       </c>
       <c r="H25" s="600" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I25" s="599" t="inlineStr">
         <is>
-          <t>전도금 입금</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J25" s="601" t="n"/>
       <c r="K25" s="601" t="n"/>
       <c r="L25" s="601" t="n"/>
       <c r="M25" s="1099" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="N25" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O25" s="1101">
@@ -44792,8 +44426,7 @@
       <c r="R25" s="1103" t="n"/>
       <c r="S25" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 여비교통비 / 판독: X)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T25" s="1097" t="n"/>
@@ -44842,10 +44475,10 @@
       <c r="K26" s="601" t="n"/>
       <c r="L26" s="601" t="n"/>
       <c r="M26" s="1099" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="N26" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O26" s="1101">
@@ -44863,8 +44496,7 @@
       <c r="R26" s="1103" t="n"/>
       <c r="S26" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 37 / 판독: 44)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T26" s="1097" t="n"/>
@@ -44913,10 +44545,10 @@
       <c r="K27" s="601" t="n"/>
       <c r="L27" s="601" t="n"/>
       <c r="M27" s="1099" t="n">
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="N27" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O27" s="1101">
@@ -44934,8 +44566,7 @@
       <c r="R27" s="1103" t="n"/>
       <c r="S27" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 36 / 판독: 37)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T27" s="1097" t="n"/>
@@ -44984,10 +44615,10 @@
       <c r="K28" s="601" t="n"/>
       <c r="L28" s="601" t="n"/>
       <c r="M28" s="1099" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="N28" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O28" s="1101">
@@ -45005,8 +44636,7 @@
       <c r="R28" s="1103" t="n"/>
       <c r="S28" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 66 / 판독: 36)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T28" s="1097" t="n"/>
@@ -45059,10 +44689,10 @@
       <c r="K29" s="601" t="n"/>
       <c r="L29" s="601" t="n"/>
       <c r="M29" s="1099" t="n">
-        <v>66</v>
+        <v>1224.6</v>
       </c>
       <c r="N29" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O29" s="1101">
@@ -45078,11 +44708,7 @@
         <v/>
       </c>
       <c r="R29" s="1103" t="n"/>
-      <c r="S29" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 44 / 판독: 66)]</t>
-        </is>
-      </c>
+      <c r="S29" s="1106" t="n"/>
       <c r="T29" s="1097" t="n"/>
       <c r="U29" s="988" t="n"/>
       <c r="V29" s="988" t="n"/>
@@ -45133,10 +44759,10 @@
       <c r="K30" s="601" t="n"/>
       <c r="L30" s="601" t="n"/>
       <c r="M30" s="1099" t="n">
-        <v>44</v>
+        <v>1019.6</v>
       </c>
       <c r="N30" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O30" s="1101">
@@ -45152,11 +44778,7 @@
         <v/>
       </c>
       <c r="R30" s="1103" t="n"/>
-      <c r="S30" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 1224.6 / 판독: 44)]</t>
-        </is>
-      </c>
+      <c r="S30" s="1106" t="n"/>
       <c r="T30" s="1097" t="n"/>
       <c r="U30" s="988" t="n"/>
       <c r="V30" s="988" t="n"/>
@@ -45203,10 +44825,10 @@
       <c r="K31" s="601" t="n"/>
       <c r="L31" s="601" t="n"/>
       <c r="M31" s="1099" t="n">
-        <v>1224.6</v>
+        <v>44</v>
       </c>
       <c r="N31" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O31" s="1101">
@@ -45224,8 +44846,7 @@
       <c r="R31" s="1103" t="n"/>
       <c r="S31" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 1019.6 / 판독: 1224.6)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T31" s="1097" t="n"/>
@@ -45266,22 +44887,22 @@
       </c>
       <c r="H32" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>해외지사비</t>
         </is>
       </c>
       <c r="I32" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J32" s="601" t="n"/>
       <c r="K32" s="601" t="n"/>
       <c r="L32" s="601" t="n"/>
       <c r="M32" s="1099" t="n">
-        <v>1019.6</v>
+        <v>198.9</v>
       </c>
       <c r="N32" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O32" s="1101">
@@ -45297,11 +44918,7 @@
         <v/>
       </c>
       <c r="R32" s="1103" t="n"/>
-      <c r="S32" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 44 / 판독: 1019.6)]</t>
-        </is>
-      </c>
+      <c r="S32" s="1106" t="n"/>
       <c r="T32" s="1097" t="n"/>
       <c r="U32" s="988" t="n"/>
       <c r="V32" s="988" t="n"/>
@@ -45340,22 +44957,22 @@
       </c>
       <c r="H33" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>해외지사비</t>
         </is>
       </c>
       <c r="I33" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J33" s="601" t="n"/>
       <c r="K33" s="601" t="n"/>
       <c r="L33" s="601" t="n"/>
       <c r="M33" s="1099" t="n">
-        <v>44</v>
+        <v>176</v>
       </c>
       <c r="N33" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O33" s="1101">
@@ -45371,12 +44988,7 @@
         <v/>
       </c>
       <c r="R33" s="1103" t="n"/>
-      <c r="S33" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 해외지사비 / 판독: 여비교통비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 198.9 / 판독: 44)]</t>
-        </is>
-      </c>
+      <c r="S33" s="1106" t="n"/>
       <c r="T33" s="1097" t="n"/>
       <c r="U33" s="988" t="n"/>
       <c r="V33" s="988" t="n"/>
@@ -45427,10 +45039,10 @@
       <c r="K34" s="601" t="n"/>
       <c r="L34" s="601" t="n"/>
       <c r="M34" s="1099" t="n">
-        <v>198.9</v>
+        <v>176</v>
       </c>
       <c r="N34" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O34" s="1101">
@@ -45446,11 +45058,7 @@
         <v/>
       </c>
       <c r="R34" s="1103" t="n"/>
-      <c r="S34" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 176 / 판독: 198.9)]</t>
-        </is>
-      </c>
+      <c r="S34" s="1106" t="n"/>
       <c r="T34" s="1097" t="n"/>
       <c r="U34" s="988" t="n"/>
       <c r="V34" s="988" t="n"/>
@@ -45501,10 +45109,10 @@
       <c r="K35" s="601" t="n"/>
       <c r="L35" s="601" t="n"/>
       <c r="M35" s="1099" t="n">
-        <v>176</v>
+        <v>197.1</v>
       </c>
       <c r="N35" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O35" s="1101">
@@ -45555,22 +45163,22 @@
       </c>
       <c r="H36" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I36" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J36" s="601" t="n"/>
       <c r="K36" s="601" t="n"/>
       <c r="L36" s="601" t="n"/>
       <c r="M36" s="1099" t="n">
-        <v>176</v>
+        <v>88</v>
       </c>
       <c r="N36" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O36" s="1101">
@@ -45588,8 +45196,7 @@
       <c r="R36" s="1103" t="n"/>
       <c r="S36" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 197.1 / 판독: 176)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T36" s="1097" t="n"/>
@@ -45626,22 +45233,22 @@
       </c>
       <c r="H37" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I37" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J37" s="601" t="n"/>
       <c r="K37" s="601" t="n"/>
       <c r="L37" s="601" t="n"/>
       <c r="M37" s="1099" t="n">
-        <v>197.1</v>
+        <v>72</v>
       </c>
       <c r="N37" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O37" s="1101">
@@ -45659,9 +45266,7 @@
       <c r="R37" s="1103" t="n"/>
       <c r="S37" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 여비교통비 / 판독: 해외지사비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 88 / 판독: 197.1)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T37" s="1097" t="n"/>
@@ -45702,22 +45307,22 @@
       </c>
       <c r="H38" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>해외지사비</t>
         </is>
       </c>
       <c r="I38" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J38" s="601" t="n"/>
       <c r="K38" s="601" t="n"/>
       <c r="L38" s="601" t="n"/>
       <c r="M38" s="1099" t="n">
-        <v>88</v>
+        <v>880</v>
       </c>
       <c r="N38" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O38" s="1101">
@@ -45733,11 +45338,7 @@
         <v/>
       </c>
       <c r="R38" s="1103" t="n"/>
-      <c r="S38" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 72 / 판독: 88)]</t>
-        </is>
-      </c>
+      <c r="S38" s="1106" t="n"/>
       <c r="T38" s="1097" t="n"/>
       <c r="U38" s="988" t="n"/>
       <c r="V38" s="988" t="n"/>
@@ -45788,10 +45389,10 @@
       <c r="K39" s="601" t="n"/>
       <c r="L39" s="601" t="n"/>
       <c r="M39" s="1099" t="n">
-        <v>72</v>
+        <v>124</v>
       </c>
       <c r="N39" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O39" s="1101">
@@ -45809,9 +45410,7 @@
       <c r="R39" s="1103" t="n"/>
       <c r="S39" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 해외지사비 / 판독: 여비교통비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 880 / 판독: 72)]
-파표 회사코드 불일치/누락</t>
+          <t>파표 회사코드 불일치/누락</t>
         </is>
       </c>
       <c r="T39" s="1097" t="n"/>
@@ -45864,10 +45463,10 @@
       <c r="K40" s="601" t="n"/>
       <c r="L40" s="601" t="n"/>
       <c r="M40" s="1099" t="n">
-        <v>880</v>
+        <v>132.36</v>
       </c>
       <c r="N40" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O40" s="1101">
@@ -45883,12 +45482,7 @@
         <v/>
       </c>
       <c r="R40" s="1103" t="n"/>
-      <c r="S40" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 여비교통비 / 판독: 해외지사비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 124 / 판독: 880)]</t>
-        </is>
-      </c>
+      <c r="S40" s="1106" t="n"/>
       <c r="T40" s="1097" t="n"/>
       <c r="U40" s="988" t="n"/>
       <c r="V40" s="988" t="n"/>
@@ -45939,10 +45533,10 @@
       <c r="K41" s="601" t="n"/>
       <c r="L41" s="601" t="n"/>
       <c r="M41" s="1099" t="n">
-        <v>124</v>
+        <v>1804</v>
       </c>
       <c r="N41" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O41" s="1101">
@@ -45958,12 +45552,7 @@
         <v/>
       </c>
       <c r="R41" s="1103" t="n"/>
-      <c r="S41" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 해외지사비 / 판독: 여비교통비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 132.36 / 판독: 124)]</t>
-        </is>
-      </c>
+      <c r="S41" s="1106" t="n"/>
       <c r="T41" s="1097" t="n"/>
       <c r="U41" s="988" t="n"/>
       <c r="V41" s="988" t="n"/>
@@ -46002,22 +45591,22 @@
       </c>
       <c r="H42" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I42" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J42" s="601" t="n"/>
       <c r="K42" s="601" t="n"/>
       <c r="L42" s="601" t="n"/>
       <c r="M42" s="1099" t="n">
-        <v>132.36</v>
+        <v>589.9</v>
       </c>
       <c r="N42" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O42" s="1101">
@@ -46033,12 +45622,7 @@
         <v/>
       </c>
       <c r="R42" s="1103" t="n"/>
-      <c r="S42" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 여비교통비 / 판독: 해외지사비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 1804 / 판독: 132.36)]</t>
-        </is>
-      </c>
+      <c r="S42" s="1106" t="n"/>
       <c r="T42" s="1097" t="n"/>
       <c r="U42" s="988" t="n"/>
       <c r="V42" s="988" t="n"/>
@@ -46085,10 +45669,10 @@
       <c r="K43" s="601" t="n"/>
       <c r="L43" s="601" t="n"/>
       <c r="M43" s="1099" t="n">
-        <v>1804</v>
+        <v>16.6</v>
       </c>
       <c r="N43" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O43" s="1101">
@@ -46106,8 +45690,7 @@
       <c r="R43" s="1103" t="n"/>
       <c r="S43" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 589.9 / 판독: 1804)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T43" s="1097" t="n"/>
@@ -46160,10 +45743,10 @@
       <c r="K44" s="601" t="n"/>
       <c r="L44" s="601" t="n"/>
       <c r="M44" s="1099" t="n">
-        <v>589.9</v>
+        <v>1824</v>
       </c>
       <c r="N44" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O44" s="1101">
@@ -46179,11 +45762,7 @@
         <v/>
       </c>
       <c r="R44" s="1103" t="n"/>
-      <c r="S44" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 16.6 / 판독: 589.9)]</t>
-        </is>
-      </c>
+      <c r="S44" s="1106" t="n"/>
       <c r="T44" s="1097" t="n"/>
       <c r="U44" s="988" t="n"/>
       <c r="V44" s="988" t="n"/>
@@ -46234,10 +45813,10 @@
       <c r="K45" s="601" t="n"/>
       <c r="L45" s="601" t="n"/>
       <c r="M45" s="1099" t="n">
-        <v>16.6</v>
+        <v>63</v>
       </c>
       <c r="N45" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O45" s="1101">
@@ -46253,11 +45832,7 @@
         <v/>
       </c>
       <c r="R45" s="1103" t="n"/>
-      <c r="S45" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 1824 / 판독: 16.6)]</t>
-        </is>
-      </c>
+      <c r="S45" s="1106" t="n"/>
       <c r="T45" s="1097" t="n"/>
       <c r="U45" s="988" t="n"/>
       <c r="V45" s="988" t="n"/>
@@ -46308,10 +45883,10 @@
       <c r="K46" s="601" t="n"/>
       <c r="L46" s="601" t="n"/>
       <c r="M46" s="1099" t="n">
-        <v>1824</v>
+        <v>887.8</v>
       </c>
       <c r="N46" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O46" s="1101">
@@ -46327,11 +45902,7 @@
         <v/>
       </c>
       <c r="R46" s="1103" t="n"/>
-      <c r="S46" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 63 / 판독: 1824)]</t>
-        </is>
-      </c>
+      <c r="S46" s="1106" t="n"/>
       <c r="T46" s="1097" t="n"/>
       <c r="U46" s="988" t="n"/>
       <c r="V46" s="988" t="n"/>
@@ -46382,10 +45953,10 @@
       <c r="K47" s="601" t="n"/>
       <c r="L47" s="601" t="n"/>
       <c r="M47" s="1099" t="n">
-        <v>63</v>
+        <v>1374</v>
       </c>
       <c r="N47" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O47" s="1101">
@@ -46401,11 +45972,7 @@
         <v/>
       </c>
       <c r="R47" s="1103" t="n"/>
-      <c r="S47" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 887.8 / 판독: 63)]</t>
-        </is>
-      </c>
+      <c r="S47" s="1106" t="n"/>
       <c r="T47" s="1097" t="n"/>
       <c r="U47" s="988" t="n"/>
       <c r="V47" s="988" t="n"/>
@@ -46456,10 +46023,10 @@
       <c r="K48" s="601" t="n"/>
       <c r="L48" s="601" t="n"/>
       <c r="M48" s="1099" t="n">
-        <v>887.8</v>
+        <v>394.5</v>
       </c>
       <c r="N48" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O48" s="1101">
@@ -46475,11 +46042,7 @@
         <v/>
       </c>
       <c r="R48" s="1103" t="n"/>
-      <c r="S48" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 1374 / 판독: 887.8)]</t>
-        </is>
-      </c>
+      <c r="S48" s="1106" t="n"/>
       <c r="T48" s="1097" t="n"/>
       <c r="U48" s="988" t="n"/>
       <c r="V48" s="988" t="n"/>
@@ -46518,22 +46081,18 @@
       </c>
       <c r="H49" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
-        </is>
-      </c>
-      <c r="I49" s="599" t="inlineStr">
-        <is>
-          <t>해외</t>
-        </is>
-      </c>
+          <t>해외지사비</t>
+        </is>
+      </c>
+      <c r="I49" s="599" t="n"/>
       <c r="J49" s="601" t="n"/>
       <c r="K49" s="601" t="n"/>
       <c r="L49" s="601" t="n"/>
       <c r="M49" s="1099" t="n">
-        <v>1374</v>
+        <v>40</v>
       </c>
       <c r="N49" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O49" s="1101">
@@ -46549,11 +46108,7 @@
         <v/>
       </c>
       <c r="R49" s="1103" t="n"/>
-      <c r="S49" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 394.5 / 판독: 1374)]</t>
-        </is>
-      </c>
+      <c r="S49" s="1106" t="n"/>
       <c r="T49" s="1097" t="n"/>
       <c r="U49" s="988" t="n"/>
       <c r="V49" s="988" t="n"/>
@@ -46604,10 +46159,10 @@
       <c r="K50" s="601" t="n"/>
       <c r="L50" s="601" t="n"/>
       <c r="M50" s="1099" t="n">
-        <v>394.5</v>
+        <v>1073</v>
       </c>
       <c r="N50" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O50" s="1101">
@@ -46623,12 +46178,7 @@
         <v/>
       </c>
       <c r="R50" s="1103" t="n"/>
-      <c r="S50" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 해외지사비 / 판독: 여비교통비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 40 / 판독: 394.5)]</t>
-        </is>
-      </c>
+      <c r="S50" s="1106" t="n"/>
       <c r="T50" s="1097" t="n"/>
       <c r="U50" s="988" t="n"/>
       <c r="V50" s="988" t="n"/>
@@ -46667,18 +46217,22 @@
       </c>
       <c r="H51" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
-        </is>
-      </c>
-      <c r="I51" s="599" t="n"/>
+          <t>여비교통비</t>
+        </is>
+      </c>
+      <c r="I51" s="599" t="inlineStr">
+        <is>
+          <t>해외</t>
+        </is>
+      </c>
       <c r="J51" s="601" t="n"/>
       <c r="K51" s="601" t="n"/>
       <c r="L51" s="601" t="n"/>
       <c r="M51" s="1099" t="n">
-        <v>40</v>
+        <v>1359</v>
       </c>
       <c r="N51" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O51" s="1101">
@@ -46694,12 +46248,7 @@
         <v/>
       </c>
       <c r="R51" s="1103" t="n"/>
-      <c r="S51" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 여비교통비 / 판독: 해외지사비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 1073 / 판독: 40)]</t>
-        </is>
-      </c>
+      <c r="S51" s="1106" t="n"/>
       <c r="T51" s="1097" t="n"/>
       <c r="U51" s="988" t="n"/>
       <c r="V51" s="988" t="n"/>
@@ -46750,10 +46299,10 @@
       <c r="K52" s="601" t="n"/>
       <c r="L52" s="601" t="n"/>
       <c r="M52" s="1099" t="n">
-        <v>1073</v>
+        <v>81.2</v>
       </c>
       <c r="N52" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O52" s="1101">
@@ -46769,11 +46318,7 @@
         <v/>
       </c>
       <c r="R52" s="1103" t="n"/>
-      <c r="S52" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 1359 / 판독: 1073)]</t>
-        </is>
-      </c>
+      <c r="S52" s="1106" t="n"/>
       <c r="T52" s="1097" t="n"/>
       <c r="U52" s="988" t="n"/>
       <c r="V52" s="988" t="n"/>
@@ -46812,22 +46357,22 @@
       </c>
       <c r="H53" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>해외지사비</t>
         </is>
       </c>
       <c r="I53" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J53" s="601" t="n"/>
       <c r="K53" s="601" t="n"/>
       <c r="L53" s="601" t="n"/>
       <c r="M53" s="1099" t="n">
-        <v>1359</v>
+        <v>378</v>
       </c>
       <c r="N53" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O53" s="1101">
@@ -46843,11 +46388,7 @@
         <v/>
       </c>
       <c r="R53" s="1103" t="n"/>
-      <c r="S53" s="1105" t="inlineStr">
-        <is>
-          <t>[⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 81.2 / 판독: 1359)]</t>
-        </is>
-      </c>
+      <c r="S53" s="1106" t="n"/>
       <c r="T53" s="1097" t="n"/>
       <c r="U53" s="988" t="n"/>
       <c r="V53" s="988" t="n"/>
@@ -46886,22 +46427,22 @@
       </c>
       <c r="H54" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>통신비</t>
         </is>
       </c>
       <c r="I54" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J54" s="601" t="n"/>
       <c r="K54" s="601" t="n"/>
       <c r="L54" s="601" t="n"/>
       <c r="M54" s="1099" t="n">
-        <v>81.2</v>
+        <v>300</v>
       </c>
       <c r="N54" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O54" s="1101">
@@ -46919,9 +46460,7 @@
       <c r="R54" s="1103" t="n"/>
       <c r="S54" s="1104" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 해외지사비 / 판독: 여비교통비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 378 / 판독: 81.2)]
-✅ 통신비 - 파표 회사코드 X</t>
+          <t>✅ 통신비 - 파표 회사코드 X</t>
         </is>
       </c>
       <c r="T54" s="1097" t="n"/>
@@ -46950,22 +46489,22 @@
       </c>
       <c r="H55" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I55" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J55" s="601" t="n"/>
       <c r="K55" s="601" t="n"/>
       <c r="L55" s="601" t="n"/>
       <c r="M55" s="1099" t="n">
-        <v>378</v>
+        <v>149</v>
       </c>
       <c r="N55" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O55" s="1101">
@@ -46983,9 +46522,7 @@
       <c r="R55" s="1103" t="n"/>
       <c r="S55" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 통신비 / 판독: 해외지사비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 300 / 판독: 378)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T55" s="1097" t="n"/>
@@ -47014,22 +46551,22 @@
       </c>
       <c r="H56" s="600" t="inlineStr">
         <is>
-          <t>통신비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I56" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J56" s="601" t="n"/>
       <c r="K56" s="601" t="n"/>
       <c r="L56" s="601" t="n"/>
       <c r="M56" s="1099" t="n">
-        <v>300</v>
+        <v>149</v>
       </c>
       <c r="N56" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O56" s="1101">
@@ -47047,9 +46584,7 @@
       <c r="R56" s="1103" t="n"/>
       <c r="S56" s="1105" t="inlineStr">
         <is>
-          <t>[⚠️ [파일명 교차검증 오류] 대계정 불일치 (파일명: 여비교통비 / 판독: 통신비)
-⚠️ [파일명 교차검증 오류] 금액 불일치 (파일명: 149 / 판독: 300)]
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T56" s="1097" t="n"/>
@@ -47063,11 +46598,7 @@
       <c r="B57" s="1098" t="n"/>
       <c r="C57" s="1098" t="n"/>
       <c r="D57" s="1098" t="inlineStr"/>
-      <c r="E57" s="306" t="inlineStr">
-        <is>
-          <t>톨비/주차비</t>
-        </is>
-      </c>
+      <c r="E57" s="306" t="n"/>
       <c r="F57" s="598" t="inlineStr">
         <is>
           <t>Lin Wei Jian</t>
@@ -47090,10 +46621,10 @@
       <c r="K57" s="601" t="n"/>
       <c r="L57" s="601" t="n"/>
       <c r="M57" s="1099" t="n">
-        <v>149</v>
+        <v>102.7</v>
       </c>
       <c r="N57" s="1100">
-        <f>'통장내역(환율표)'!$D$88</f>
+        <f>'통장내역(환율표)'!D94</f>
         <v/>
       </c>
       <c r="O57" s="1101">
@@ -52795,7 +52326,6 @@
     <brk id="11" min="0" max="1048575" man="1"/>
     <brk id="13" min="0" max="1048575" man="1"/>
   </colBreaks>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -52958,12 +52488,12 @@
       <c r="G2" s="1108" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="643" t="inlineStr">
+      <c r="B4" s="650" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
-      <c r="C4" s="643" t="inlineStr">
+      <c r="C4" s="650" t="inlineStr">
         <is>
           <t>정산일자</t>
         </is>
@@ -52983,23 +52513,23 @@
           <t>사용처</t>
         </is>
       </c>
-      <c r="G4" s="643" t="inlineStr">
+      <c r="G4" s="650" t="inlineStr">
         <is>
           <t>사용금액</t>
         </is>
       </c>
       <c r="H4" s="1110" t="n"/>
-      <c r="I4" s="643" t="inlineStr">
+      <c r="I4" s="650" t="inlineStr">
         <is>
           <t>사용목적(상세 기재)</t>
         </is>
       </c>
-      <c r="J4" s="643" t="inlineStr">
+      <c r="J4" s="650" t="inlineStr">
         <is>
           <t>고객명</t>
         </is>
       </c>
-      <c r="K4" s="643" t="inlineStr">
+      <c r="K4" s="650" t="inlineStr">
         <is>
           <t>참석자</t>
         </is>
@@ -53017,19 +52547,19 @@
           <t>RMB</t>
         </is>
       </c>
-      <c r="H5" s="643" t="inlineStr">
+      <c r="H5" s="650" t="inlineStr">
         <is>
           <t>KRW</t>
         </is>
       </c>
       <c r="I5" s="1111" t="n"/>
       <c r="J5" s="1111" t="n"/>
-      <c r="K5" s="643" t="inlineStr">
+      <c r="K5" s="650" t="inlineStr">
         <is>
           <t>고객</t>
         </is>
       </c>
-      <c r="L5" s="643" t="inlineStr">
+      <c r="L5" s="650" t="inlineStr">
         <is>
           <t>DBGC</t>
         </is>

</xml_diff>

<commit_message>
Refactor: Update batch_processor and app.py to support nested account subdirectories and cross-check folder names
</commit_message>
<xml_diff>
--- a/작업장소 (영수증 보관)/2026-06/심천지사 전도금 정산 양식_2026-06.xlsx
+++ b/작업장소 (영수증 보관)/2026-06/심천지사 전도금 정산 양식_2026-06.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="603" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11295" tabRatio="603" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="통장내역(환율표)" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="내역_25.01" sheetId="2" state="hidden" r:id="rId2"/>
-    <sheet name="내역_25.02" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet name="내역_25.03" sheetId="4" state="hidden" r:id="rId4"/>
-    <sheet name="내역_25.04" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet name="내역_25.05" sheetId="6" state="hidden" r:id="rId6"/>
-    <sheet name="2026-06" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="통장지급내역" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="당월 업무추진비" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="기사 야근 일지" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통장내역(환율표)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="내역_25.01" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="내역_25.02" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="내역_25.03" sheetId="4" state="hidden" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="내역_25.04" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="내역_25.05" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026-06" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="통장지급내역" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="당월 업무추진비" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기사 야근 일지" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId11"/>
-    <externalReference r:id="rId12"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId11"/>
+    <externalReference xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId12"/>
   </externalReferences>
   <definedNames>
     <definedName name="Large_scale_classification">[1]Sheet3!$C$4:$C$10</definedName>
@@ -6565,14 +6565,14 @@
     <xf numFmtId="167" fontId="12" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
       <alignment vertical="center" shrinkToFit="1"/>
     </xf>
+    <xf numFmtId="167" fontId="87" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="87" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="27" applyAlignment="1" pivotButton="0" quotePrefix="1" xfId="138">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
     <xf numFmtId="166" fontId="65" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="177">
       <alignment vertical="center"/>
@@ -7391,8 +7391,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Report"/>
       <sheetName val="classification"/>
@@ -7448,8 +7448,8 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <externalBook r:id="rId1">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="통장내역(환율표)"/>
       <sheetName val="내역_22.03"/>
@@ -11259,7 +11259,7 @@
       <c r="F2" s="701" t="n"/>
       <c r="G2" s="688" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H2" s="206" t="inlineStr">
@@ -17662,7 +17662,7 @@
       <c r="F2" s="701" t="n"/>
       <c r="G2" s="688" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H2" s="206" t="inlineStr">
@@ -23470,7 +23470,7 @@
       <c r="F2" s="701" t="n"/>
       <c r="G2" s="688" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H2" s="206" t="inlineStr">
@@ -29866,7 +29866,7 @@
       <c r="F2" s="701" t="n"/>
       <c r="G2" s="688" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H2" s="206" t="inlineStr">
@@ -36373,7 +36373,7 @@
       <c r="F2" s="701" t="n"/>
       <c r="G2" s="688" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H2" s="206" t="inlineStr">
@@ -43229,14 +43229,14 @@
   <mergeCells count="11">
     <mergeCell ref="N17:O17"/>
     <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="R94:R98"/>
     <mergeCell ref="P17:Q17"/>
     <mergeCell ref="R79:R83"/>
-    <mergeCell ref="R103:R107"/>
     <mergeCell ref="R84:R88"/>
     <mergeCell ref="R89:R93"/>
     <mergeCell ref="K17:M17"/>
     <mergeCell ref="H17:J17"/>
-    <mergeCell ref="R94:R98"/>
+    <mergeCell ref="R103:R107"/>
     <mergeCell ref="R99:R102"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -43308,7 +43308,7 @@
       <c r="F2" s="1002" t="n"/>
       <c r="G2" s="989" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
       <c r="H2" s="445" t="inlineStr">
@@ -44162,23 +44162,23 @@
       <c r="A22" s="537" t="n"/>
       <c r="B22" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="C22" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="D22" s="1098" t="inlineStr"/>
       <c r="E22" s="306" t="inlineStr">
         <is>
-          <t>USD입금/RMB환전 CNY 505742.12</t>
+          <t>톨비/주차비</t>
         </is>
       </c>
       <c r="F22" s="598" t="inlineStr">
         <is>
-          <t>심천지사</t>
+          <t>Lin Wei Jian</t>
         </is>
       </c>
       <c r="G22" s="599" t="n">
@@ -44186,26 +44186,28 @@
       </c>
       <c r="H22" s="600" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I22" s="599" t="inlineStr">
         <is>
-          <t>전도금 입금</t>
-        </is>
-      </c>
-      <c r="J22" s="601" t="n">
-        <v>505742.12</v>
-      </c>
-      <c r="K22" s="601" t="n">
-        <v>6.7491</v>
-      </c>
-      <c r="L22" s="601" t="n">
-        <v>74959.75</v>
-      </c>
-      <c r="M22" s="1099" t="n"/>
-      <c r="N22" s="1100" t="n"/>
-      <c r="O22" s="1101" t="inlineStr"/>
+          <t>해외</t>
+        </is>
+      </c>
+      <c r="J22" s="601" t="n"/>
+      <c r="K22" s="601" t="n"/>
+      <c r="L22" s="601" t="n"/>
+      <c r="M22" s="1099" t="n">
+        <v>44</v>
+      </c>
+      <c r="N22" s="1100">
+        <f>'통장내역(환율표)'!D94</f>
+        <v/>
+      </c>
+      <c r="O22" s="1101">
+        <f>M22/N22</f>
+        <v/>
+      </c>
       <c r="P22" s="1102">
         <f>P21+J22-M22</f>
         <v/>
@@ -44217,8 +44219,7 @@
       <c r="R22" s="1103" t="n"/>
       <c r="S22" s="1104" t="inlineStr">
         <is>
-          <t>✅ 입금 확인 (USD: 74959.75 / 환산요율: 6.7491 / 수수료 USD: 25)
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T22" s="1097" t="n"/>
@@ -44231,48 +44232,51 @@
       <c r="A23" s="537" t="n"/>
       <c r="B23" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="C23" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="D23" s="1098" t="inlineStr"/>
       <c r="E23" s="306" t="inlineStr">
         <is>
-          <t>USD입금/RMB환전 수수료 USD 25</t>
+          <t>톨비/주차비</t>
         </is>
       </c>
       <c r="F23" s="598" t="inlineStr">
         <is>
-          <t>심천지사</t>
+          <t>Lin Wei Jian</t>
         </is>
       </c>
       <c r="G23" s="599" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H23" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I23" s="599" t="inlineStr">
         <is>
-          <t>전도금 입금</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J23" s="601" t="n"/>
       <c r="K23" s="601" t="n"/>
       <c r="L23" s="601" t="n"/>
-      <c r="M23" s="1099">
-        <f>O23*N23</f>
-        <v/>
-      </c>
-      <c r="N23" s="1100" t="n"/>
-      <c r="O23" s="1101" t="n">
-        <v>25</v>
+      <c r="M23" s="1099" t="n">
+        <v>37</v>
+      </c>
+      <c r="N23" s="1100">
+        <f>'통장내역(환율표)'!D94</f>
+        <v/>
+      </c>
+      <c r="O23" s="1101">
+        <f>M23/N23</f>
+        <v/>
       </c>
       <c r="P23" s="1102">
         <f>P22+J23-M23</f>
@@ -44285,8 +44289,7 @@
       <c r="R23" s="1103" t="n"/>
       <c r="S23" s="1104" t="inlineStr">
         <is>
-          <t>✅ 입금 확인 (USD: 74959.75 / 환산요율: 6.7491 / 수수료 USD: 25)
-파표 외 영수증</t>
+          <t>파표 외 영수증</t>
         </is>
       </c>
       <c r="T23" s="1097" t="n"/>
@@ -44299,12 +44302,12 @@
       <c r="A24" s="537" t="n"/>
       <c r="B24" s="1098" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="C24" s="1098" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="D24" s="1098" t="inlineStr"/>
@@ -44319,7 +44322,7 @@
         </is>
       </c>
       <c r="G24" s="599" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" s="600" t="inlineStr">
         <is>
@@ -44335,7 +44338,7 @@
       <c r="K24" s="601" t="n"/>
       <c r="L24" s="601" t="n"/>
       <c r="M24" s="1099" t="n">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="N24" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44354,7 +44357,7 @@
         <v/>
       </c>
       <c r="R24" s="1103" t="n"/>
-      <c r="S24" s="1105" t="inlineStr">
+      <c r="S24" s="1104" t="inlineStr">
         <is>
           <t>파표 외 영수증</t>
         </is>
@@ -44369,12 +44372,12 @@
       <c r="A25" s="537" t="n"/>
       <c r="B25" s="1098" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="C25" s="1098" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-05-06</t>
         </is>
       </c>
       <c r="D25" s="1098" t="inlineStr"/>
@@ -44389,7 +44392,7 @@
         </is>
       </c>
       <c r="G25" s="599" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H25" s="600" t="inlineStr">
         <is>
@@ -44405,7 +44408,7 @@
       <c r="K25" s="601" t="n"/>
       <c r="L25" s="601" t="n"/>
       <c r="M25" s="1099" t="n">
-        <v>37</v>
+        <v>66</v>
       </c>
       <c r="N25" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44424,7 +44427,7 @@
         <v/>
       </c>
       <c r="R25" s="1103" t="n"/>
-      <c r="S25" s="1105" t="inlineStr">
+      <c r="S25" s="1104" t="inlineStr">
         <is>
           <t>파표 외 영수증</t>
         </is>
@@ -44439,12 +44442,12 @@
       <c r="A26" s="537" t="n"/>
       <c r="B26" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C26" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D26" s="1098" t="inlineStr"/>
@@ -44459,7 +44462,7 @@
         </is>
       </c>
       <c r="G26" s="599" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H26" s="600" t="inlineStr">
         <is>
@@ -44475,7 +44478,7 @@
       <c r="K26" s="601" t="n"/>
       <c r="L26" s="601" t="n"/>
       <c r="M26" s="1099" t="n">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="N26" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44494,7 +44497,7 @@
         <v/>
       </c>
       <c r="R26" s="1103" t="n"/>
-      <c r="S26" s="1105" t="inlineStr">
+      <c r="S26" s="1104" t="inlineStr">
         <is>
           <t>파표 외 영수증</t>
         </is>
@@ -44509,18 +44512,22 @@
       <c r="A27" s="537" t="n"/>
       <c r="B27" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C27" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
-        </is>
-      </c>
-      <c r="D27" s="1098" t="inlineStr"/>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="D27" s="1098" t="inlineStr">
+        <is>
+          <t>26957000000133687853</t>
+        </is>
+      </c>
       <c r="E27" s="306" t="inlineStr">
         <is>
-          <t>톨비/주차비</t>
+          <t>교통비</t>
         </is>
       </c>
       <c r="F27" s="598" t="inlineStr">
@@ -44529,7 +44536,7 @@
         </is>
       </c>
       <c r="G27" s="599" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H27" s="600" t="inlineStr">
         <is>
@@ -44545,7 +44552,7 @@
       <c r="K27" s="601" t="n"/>
       <c r="L27" s="601" t="n"/>
       <c r="M27" s="1099" t="n">
-        <v>66</v>
+        <v>1224.6</v>
       </c>
       <c r="N27" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44564,11 +44571,7 @@
         <v/>
       </c>
       <c r="R27" s="1103" t="n"/>
-      <c r="S27" s="1105" t="inlineStr">
-        <is>
-          <t>파표 외 영수증</t>
-        </is>
-      </c>
+      <c r="S27" s="1105" t="n"/>
       <c r="T27" s="1097" t="n"/>
       <c r="U27" s="988" t="n"/>
       <c r="V27" s="988" t="n"/>
@@ -44579,18 +44582,22 @@
       <c r="A28" s="537" t="n"/>
       <c r="B28" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C28" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
-      <c r="D28" s="1098" t="inlineStr"/>
+          <t>2026-05-19</t>
+        </is>
+      </c>
+      <c r="D28" s="1098" t="inlineStr">
+        <is>
+          <t>26447000001043120863</t>
+        </is>
+      </c>
       <c r="E28" s="306" t="inlineStr">
         <is>
-          <t>톨비/주차비</t>
+          <t>교통비</t>
         </is>
       </c>
       <c r="F28" s="598" t="inlineStr">
@@ -44599,7 +44606,7 @@
         </is>
       </c>
       <c r="G28" s="599" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H28" s="600" t="inlineStr">
         <is>
@@ -44615,7 +44622,7 @@
       <c r="K28" s="601" t="n"/>
       <c r="L28" s="601" t="n"/>
       <c r="M28" s="1099" t="n">
-        <v>44</v>
+        <v>1019.6</v>
       </c>
       <c r="N28" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44634,11 +44641,7 @@
         <v/>
       </c>
       <c r="R28" s="1103" t="n"/>
-      <c r="S28" s="1105" t="inlineStr">
-        <is>
-          <t>파표 외 영수증</t>
-        </is>
-      </c>
+      <c r="S28" s="1105" t="n"/>
       <c r="T28" s="1097" t="n"/>
       <c r="U28" s="988" t="n"/>
       <c r="V28" s="988" t="n"/>
@@ -44649,22 +44652,18 @@
       <c r="A29" s="537" t="n"/>
       <c r="B29" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C29" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="D29" s="1098" t="inlineStr">
-        <is>
-          <t>26957000000133687853</t>
-        </is>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="D29" s="1098" t="inlineStr"/>
       <c r="E29" s="306" t="inlineStr">
         <is>
-          <t>교통비</t>
+          <t>톨비/주차비</t>
         </is>
       </c>
       <c r="F29" s="598" t="inlineStr">
@@ -44673,7 +44672,7 @@
         </is>
       </c>
       <c r="G29" s="599" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H29" s="600" t="inlineStr">
         <is>
@@ -44689,7 +44688,7 @@
       <c r="K29" s="601" t="n"/>
       <c r="L29" s="601" t="n"/>
       <c r="M29" s="1099" t="n">
-        <v>1224.6</v>
+        <v>44</v>
       </c>
       <c r="N29" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44708,7 +44707,11 @@
         <v/>
       </c>
       <c r="R29" s="1103" t="n"/>
-      <c r="S29" s="1106" t="n"/>
+      <c r="S29" s="1104" t="inlineStr">
+        <is>
+          <t>파표 외 영수증</t>
+        </is>
+      </c>
       <c r="T29" s="1097" t="n"/>
       <c r="U29" s="988" t="n"/>
       <c r="V29" s="988" t="n"/>
@@ -44719,22 +44722,18 @@
       <c r="A30" s="537" t="n"/>
       <c r="B30" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C30" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="D30" s="1098" t="inlineStr">
-        <is>
-          <t>26447000001043120863</t>
-        </is>
-      </c>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="D30" s="1098" t="inlineStr"/>
       <c r="E30" s="306" t="inlineStr">
         <is>
-          <t>교통비</t>
+          <t>톨비/주차비</t>
         </is>
       </c>
       <c r="F30" s="598" t="inlineStr">
@@ -44743,7 +44742,7 @@
         </is>
       </c>
       <c r="G30" s="599" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H30" s="600" t="inlineStr">
         <is>
@@ -44759,7 +44758,7 @@
       <c r="K30" s="601" t="n"/>
       <c r="L30" s="601" t="n"/>
       <c r="M30" s="1099" t="n">
-        <v>1019.6</v>
+        <v>44</v>
       </c>
       <c r="N30" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44778,7 +44777,12 @@
         <v/>
       </c>
       <c r="R30" s="1103" t="n"/>
-      <c r="S30" s="1106" t="n"/>
+      <c r="S30" s="1104" t="inlineStr">
+        <is>
+          <t>[⚠️ 이번 달 14번 영수증과 중복 (증빙/주문번호: 41185202605224045313201121582)]
+파표 외 영수증</t>
+        </is>
+      </c>
       <c r="T30" s="1097" t="n"/>
       <c r="U30" s="988" t="n"/>
       <c r="V30" s="988" t="n"/>
@@ -44789,18 +44793,22 @@
       <c r="A31" s="537" t="n"/>
       <c r="B31" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="C31" s="1098" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
-        </is>
-      </c>
-      <c r="D31" s="1098" t="inlineStr"/>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="D31" s="1098" t="inlineStr">
+        <is>
+          <t>26957000000141421480</t>
+        </is>
+      </c>
       <c r="E31" s="306" t="inlineStr">
         <is>
-          <t>톨비/주차비</t>
+          <t>택배비</t>
         </is>
       </c>
       <c r="F31" s="598" t="inlineStr">
@@ -44809,23 +44817,23 @@
         </is>
       </c>
       <c r="G31" s="599" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H31" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>해외지사비</t>
         </is>
       </c>
       <c r="I31" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J31" s="601" t="n"/>
       <c r="K31" s="601" t="n"/>
       <c r="L31" s="601" t="n"/>
       <c r="M31" s="1099" t="n">
-        <v>44</v>
+        <v>176</v>
       </c>
       <c r="N31" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44844,11 +44852,7 @@
         <v/>
       </c>
       <c r="R31" s="1103" t="n"/>
-      <c r="S31" s="1105" t="inlineStr">
-        <is>
-          <t>파표 외 영수증</t>
-        </is>
-      </c>
+      <c r="S31" s="1105" t="n"/>
       <c r="T31" s="1097" t="n"/>
       <c r="U31" s="988" t="n"/>
       <c r="V31" s="988" t="n"/>
@@ -44869,7 +44873,7 @@
       </c>
       <c r="D32" s="1098" t="inlineStr">
         <is>
-          <t>26957000000141421482</t>
+          <t>26957000000141421481</t>
         </is>
       </c>
       <c r="E32" s="306" t="inlineStr">
@@ -44883,7 +44887,7 @@
         </is>
       </c>
       <c r="G32" s="599" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H32" s="600" t="inlineStr">
         <is>
@@ -44899,7 +44903,7 @@
       <c r="K32" s="601" t="n"/>
       <c r="L32" s="601" t="n"/>
       <c r="M32" s="1099" t="n">
-        <v>198.9</v>
+        <v>176</v>
       </c>
       <c r="N32" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44918,7 +44922,7 @@
         <v/>
       </c>
       <c r="R32" s="1103" t="n"/>
-      <c r="S32" s="1106" t="n"/>
+      <c r="S32" s="1105" t="n"/>
       <c r="T32" s="1097" t="n"/>
       <c r="U32" s="988" t="n"/>
       <c r="V32" s="988" t="n"/>
@@ -44939,7 +44943,7 @@
       </c>
       <c r="D33" s="1098" t="inlineStr">
         <is>
-          <t>26957000000141421480</t>
+          <t>26957000000141421482</t>
         </is>
       </c>
       <c r="E33" s="306" t="inlineStr">
@@ -44953,7 +44957,7 @@
         </is>
       </c>
       <c r="G33" s="599" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H33" s="600" t="inlineStr">
         <is>
@@ -44969,7 +44973,7 @@
       <c r="K33" s="601" t="n"/>
       <c r="L33" s="601" t="n"/>
       <c r="M33" s="1099" t="n">
-        <v>176</v>
+        <v>198.9</v>
       </c>
       <c r="N33" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -44988,7 +44992,7 @@
         <v/>
       </c>
       <c r="R33" s="1103" t="n"/>
-      <c r="S33" s="1106" t="n"/>
+      <c r="S33" s="1105" t="n"/>
       <c r="T33" s="1097" t="n"/>
       <c r="U33" s="988" t="n"/>
       <c r="V33" s="988" t="n"/>
@@ -45009,7 +45013,7 @@
       </c>
       <c r="D34" s="1098" t="inlineStr">
         <is>
-          <t>26957000000141421481</t>
+          <t>26957000000141421483</t>
         </is>
       </c>
       <c r="E34" s="306" t="inlineStr">
@@ -45023,7 +45027,7 @@
         </is>
       </c>
       <c r="G34" s="599" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H34" s="600" t="inlineStr">
         <is>
@@ -45039,7 +45043,7 @@
       <c r="K34" s="601" t="n"/>
       <c r="L34" s="601" t="n"/>
       <c r="M34" s="1099" t="n">
-        <v>176</v>
+        <v>197.1</v>
       </c>
       <c r="N34" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45058,7 +45062,7 @@
         <v/>
       </c>
       <c r="R34" s="1103" t="n"/>
-      <c r="S34" s="1106" t="n"/>
+      <c r="S34" s="1105" t="n"/>
       <c r="T34" s="1097" t="n"/>
       <c r="U34" s="988" t="n"/>
       <c r="V34" s="988" t="n"/>
@@ -45069,22 +45073,18 @@
       <c r="A35" s="537" t="n"/>
       <c r="B35" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-07</t>
         </is>
       </c>
       <c r="C35" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
-        </is>
-      </c>
-      <c r="D35" s="1098" t="inlineStr">
-        <is>
-          <t>26957000000141421483</t>
-        </is>
-      </c>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="D35" s="1098" t="inlineStr"/>
       <c r="E35" s="306" t="inlineStr">
         <is>
-          <t>택배비</t>
+          <t>톨비/주차비</t>
         </is>
       </c>
       <c r="F35" s="598" t="inlineStr">
@@ -45093,23 +45093,23 @@
         </is>
       </c>
       <c r="G35" s="599" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H35" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I35" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J35" s="601" t="n"/>
       <c r="K35" s="601" t="n"/>
       <c r="L35" s="601" t="n"/>
       <c r="M35" s="1099" t="n">
-        <v>197.1</v>
+        <v>88</v>
       </c>
       <c r="N35" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45128,7 +45128,11 @@
         <v/>
       </c>
       <c r="R35" s="1103" t="n"/>
-      <c r="S35" s="1106" t="n"/>
+      <c r="S35" s="1104" t="inlineStr">
+        <is>
+          <t>파표 외 영수증</t>
+        </is>
+      </c>
       <c r="T35" s="1097" t="n"/>
       <c r="U35" s="988" t="n"/>
       <c r="V35" s="988" t="n"/>
@@ -45159,7 +45163,7 @@
         </is>
       </c>
       <c r="G36" s="599" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H36" s="600" t="inlineStr">
         <is>
@@ -45194,9 +45198,10 @@
         <v/>
       </c>
       <c r="R36" s="1103" t="n"/>
-      <c r="S36" s="1105" t="inlineStr">
-        <is>
-          <t>파표 외 영수증</t>
+      <c r="S36" s="1104" t="inlineStr">
+        <is>
+          <t>[⚠️ 이번 달 19번 영수증과 중복 (증빙/주문번호: 41185202606074050639601999655)]
+파표 외 영수증</t>
         </is>
       </c>
       <c r="T36" s="1097" t="n"/>
@@ -45229,7 +45234,7 @@
         </is>
       </c>
       <c r="G37" s="599" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H37" s="600" t="inlineStr">
         <is>
@@ -45264,7 +45269,7 @@
         <v/>
       </c>
       <c r="R37" s="1103" t="n"/>
-      <c r="S37" s="1105" t="inlineStr">
+      <c r="S37" s="1104" t="inlineStr">
         <is>
           <t>파표 외 영수증</t>
         </is>
@@ -45279,22 +45284,18 @@
       <c r="A38" s="537" t="n"/>
       <c r="B38" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="C38" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
-        </is>
-      </c>
-      <c r="D38" s="1098" t="inlineStr">
-        <is>
-          <t>26952000002433520066</t>
-        </is>
-      </c>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+      <c r="D38" s="1098" t="inlineStr"/>
       <c r="E38" s="306" t="inlineStr">
         <is>
-          <t>택배비/운송비</t>
+          <t>톨비/주차비</t>
         </is>
       </c>
       <c r="F38" s="598" t="inlineStr">
@@ -45303,23 +45304,23 @@
         </is>
       </c>
       <c r="G38" s="599" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H38" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I38" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J38" s="601" t="n"/>
       <c r="K38" s="601" t="n"/>
       <c r="L38" s="601" t="n"/>
       <c r="M38" s="1099" t="n">
-        <v>880</v>
+        <v>72</v>
       </c>
       <c r="N38" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45338,7 +45339,12 @@
         <v/>
       </c>
       <c r="R38" s="1103" t="n"/>
-      <c r="S38" s="1106" t="n"/>
+      <c r="S38" s="1104" t="inlineStr">
+        <is>
+          <t>[⚠️ 이번 달 18번 영수증과 중복 (증빙/주문번호: 41185202606084051438101778823)]
+파표 외 영수증</t>
+        </is>
+      </c>
       <c r="T38" s="1097" t="n"/>
       <c r="U38" s="988" t="n"/>
       <c r="V38" s="988" t="n"/>
@@ -45349,22 +45355,22 @@
       <c r="A39" s="537" t="n"/>
       <c r="B39" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="C39" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
       <c r="D39" s="1098" t="inlineStr">
         <is>
-          <t>02474918</t>
+          <t>26952000002433520066</t>
         </is>
       </c>
       <c r="E39" s="306" t="inlineStr">
         <is>
-          <t>톨비/주차비</t>
+          <t>택배비/운송비</t>
         </is>
       </c>
       <c r="F39" s="598" t="inlineStr">
@@ -45373,23 +45379,23 @@
         </is>
       </c>
       <c r="G39" s="599" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H39" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>해외지사비</t>
         </is>
       </c>
       <c r="I39" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J39" s="601" t="n"/>
       <c r="K39" s="601" t="n"/>
       <c r="L39" s="601" t="n"/>
       <c r="M39" s="1099" t="n">
-        <v>124</v>
+        <v>880</v>
       </c>
       <c r="N39" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45408,11 +45414,7 @@
         <v/>
       </c>
       <c r="R39" s="1103" t="n"/>
-      <c r="S39" s="1105" t="inlineStr">
-        <is>
-          <t>파표 회사코드 불일치/누락</t>
-        </is>
-      </c>
+      <c r="S39" s="1105" t="n"/>
       <c r="T39" s="1097" t="n"/>
       <c r="U39" s="988" t="n"/>
       <c r="V39" s="988" t="n"/>
@@ -45423,22 +45425,22 @@
       <c r="A40" s="537" t="n"/>
       <c r="B40" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="C40" s="1098" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="D40" s="1098" t="inlineStr">
         <is>
-          <t>45212619</t>
+          <t>02474918</t>
         </is>
       </c>
       <c r="E40" s="306" t="inlineStr">
         <is>
-          <t>화물운송료</t>
+          <t>톨비/주차비</t>
         </is>
       </c>
       <c r="F40" s="598" t="inlineStr">
@@ -45447,23 +45449,23 @@
         </is>
       </c>
       <c r="G40" s="599" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H40" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I40" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J40" s="601" t="n"/>
       <c r="K40" s="601" t="n"/>
       <c r="L40" s="601" t="n"/>
       <c r="M40" s="1099" t="n">
-        <v>132.36</v>
+        <v>124</v>
       </c>
       <c r="N40" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45482,7 +45484,11 @@
         <v/>
       </c>
       <c r="R40" s="1103" t="n"/>
-      <c r="S40" s="1106" t="n"/>
+      <c r="S40" s="1104" t="inlineStr">
+        <is>
+          <t>파표 회사코드 불일치/누락</t>
+        </is>
+      </c>
       <c r="T40" s="1097" t="n"/>
       <c r="U40" s="988" t="n"/>
       <c r="V40" s="988" t="n"/>
@@ -45517,7 +45523,7 @@
         </is>
       </c>
       <c r="G41" s="599" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H41" s="600" t="inlineStr">
         <is>
@@ -45552,7 +45558,7 @@
         <v/>
       </c>
       <c r="R41" s="1103" t="n"/>
-      <c r="S41" s="1106" t="n"/>
+      <c r="S41" s="1105" t="n"/>
       <c r="T41" s="1097" t="n"/>
       <c r="U41" s="988" t="n"/>
       <c r="V41" s="988" t="n"/>
@@ -45573,12 +45579,12 @@
       </c>
       <c r="D42" s="1098" t="inlineStr">
         <is>
-          <t>26957000000165619116</t>
+          <t>26442000006669013351</t>
         </is>
       </c>
       <c r="E42" s="306" t="inlineStr">
         <is>
-          <t>교통비</t>
+          <t>숙박비</t>
         </is>
       </c>
       <c r="F42" s="598" t="inlineStr">
@@ -45587,7 +45593,7 @@
         </is>
       </c>
       <c r="G42" s="599" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H42" s="600" t="inlineStr">
         <is>
@@ -45603,7 +45609,7 @@
       <c r="K42" s="601" t="n"/>
       <c r="L42" s="601" t="n"/>
       <c r="M42" s="1099" t="n">
-        <v>589.9</v>
+        <v>1824</v>
       </c>
       <c r="N42" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45622,7 +45628,7 @@
         <v/>
       </c>
       <c r="R42" s="1103" t="n"/>
-      <c r="S42" s="1106" t="n"/>
+      <c r="S42" s="1105" t="n"/>
       <c r="T42" s="1097" t="n"/>
       <c r="U42" s="988" t="n"/>
       <c r="V42" s="988" t="n"/>
@@ -45641,10 +45647,14 @@
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="D43" s="1098" t="inlineStr"/>
+      <c r="D43" s="1098" t="inlineStr">
+        <is>
+          <t>26442000006669091216</t>
+        </is>
+      </c>
       <c r="E43" s="306" t="inlineStr">
         <is>
-          <t>항공권</t>
+          <t>숙박비</t>
         </is>
       </c>
       <c r="F43" s="598" t="inlineStr">
@@ -45653,7 +45663,7 @@
         </is>
       </c>
       <c r="G43" s="599" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H43" s="600" t="inlineStr">
         <is>
@@ -45669,7 +45679,7 @@
       <c r="K43" s="601" t="n"/>
       <c r="L43" s="601" t="n"/>
       <c r="M43" s="1099" t="n">
-        <v>16.6</v>
+        <v>1359</v>
       </c>
       <c r="N43" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45688,11 +45698,7 @@
         <v/>
       </c>
       <c r="R43" s="1103" t="n"/>
-      <c r="S43" s="1105" t="inlineStr">
-        <is>
-          <t>파표 외 영수증</t>
-        </is>
-      </c>
+      <c r="S43" s="1105" t="n"/>
       <c r="T43" s="1097" t="n"/>
       <c r="U43" s="988" t="n"/>
       <c r="V43" s="988" t="n"/>
@@ -45713,7 +45719,7 @@
       </c>
       <c r="D44" s="1098" t="inlineStr">
         <is>
-          <t>26442000006669013351</t>
+          <t>26442000006668490571</t>
         </is>
       </c>
       <c r="E44" s="306" t="inlineStr">
@@ -45727,7 +45733,7 @@
         </is>
       </c>
       <c r="G44" s="599" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H44" s="600" t="inlineStr">
         <is>
@@ -45743,7 +45749,7 @@
       <c r="K44" s="601" t="n"/>
       <c r="L44" s="601" t="n"/>
       <c r="M44" s="1099" t="n">
-        <v>1824</v>
+        <v>1374</v>
       </c>
       <c r="N44" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45762,7 +45768,7 @@
         <v/>
       </c>
       <c r="R44" s="1103" t="n"/>
-      <c r="S44" s="1106" t="n"/>
+      <c r="S44" s="1105" t="n"/>
       <c r="T44" s="1097" t="n"/>
       <c r="U44" s="988" t="n"/>
       <c r="V44" s="988" t="n"/>
@@ -45783,12 +45789,12 @@
       </c>
       <c r="D45" s="1098" t="inlineStr">
         <is>
-          <t>26327000001122217548</t>
+          <t>26517000000466701406</t>
         </is>
       </c>
       <c r="E45" s="306" t="inlineStr">
         <is>
-          <t>항공권</t>
+          <t>교통비</t>
         </is>
       </c>
       <c r="F45" s="598" t="inlineStr">
@@ -45797,7 +45803,7 @@
         </is>
       </c>
       <c r="G45" s="599" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H45" s="600" t="inlineStr">
         <is>
@@ -45813,7 +45819,7 @@
       <c r="K45" s="601" t="n"/>
       <c r="L45" s="601" t="n"/>
       <c r="M45" s="1099" t="n">
-        <v>63</v>
+        <v>394.5</v>
       </c>
       <c r="N45" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45832,7 +45838,7 @@
         <v/>
       </c>
       <c r="R45" s="1103" t="n"/>
-      <c r="S45" s="1106" t="n"/>
+      <c r="S45" s="1105" t="n"/>
       <c r="T45" s="1097" t="n"/>
       <c r="U45" s="988" t="n"/>
       <c r="V45" s="988" t="n"/>
@@ -45853,7 +45859,7 @@
       </c>
       <c r="D46" s="1098" t="inlineStr">
         <is>
-          <t>26447000001222315056</t>
+          <t>26957000000165619116</t>
         </is>
       </c>
       <c r="E46" s="306" t="inlineStr">
@@ -45867,7 +45873,7 @@
         </is>
       </c>
       <c r="G46" s="599" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H46" s="600" t="inlineStr">
         <is>
@@ -45883,7 +45889,7 @@
       <c r="K46" s="601" t="n"/>
       <c r="L46" s="601" t="n"/>
       <c r="M46" s="1099" t="n">
-        <v>887.8</v>
+        <v>589.9</v>
       </c>
       <c r="N46" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45902,7 +45908,7 @@
         <v/>
       </c>
       <c r="R46" s="1103" t="n"/>
-      <c r="S46" s="1106" t="n"/>
+      <c r="S46" s="1105" t="n"/>
       <c r="T46" s="1097" t="n"/>
       <c r="U46" s="988" t="n"/>
       <c r="V46" s="988" t="n"/>
@@ -45921,14 +45927,10 @@
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="D47" s="1098" t="inlineStr">
-        <is>
-          <t>26442000006668490571</t>
-        </is>
-      </c>
+      <c r="D47" s="1098" t="inlineStr"/>
       <c r="E47" s="306" t="inlineStr">
         <is>
-          <t>숙박비</t>
+          <t>항공권</t>
         </is>
       </c>
       <c r="F47" s="598" t="inlineStr">
@@ -45937,7 +45939,7 @@
         </is>
       </c>
       <c r="G47" s="599" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H47" s="600" t="inlineStr">
         <is>
@@ -45953,7 +45955,7 @@
       <c r="K47" s="601" t="n"/>
       <c r="L47" s="601" t="n"/>
       <c r="M47" s="1099" t="n">
-        <v>1374</v>
+        <v>16.6</v>
       </c>
       <c r="N47" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -45972,7 +45974,11 @@
         <v/>
       </c>
       <c r="R47" s="1103" t="n"/>
-      <c r="S47" s="1106" t="n"/>
+      <c r="S47" s="1104" t="inlineStr">
+        <is>
+          <t>파표 외 영수증</t>
+        </is>
+      </c>
       <c r="T47" s="1097" t="n"/>
       <c r="U47" s="988" t="n"/>
       <c r="V47" s="988" t="n"/>
@@ -46007,7 +46013,7 @@
         </is>
       </c>
       <c r="G48" s="599" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H48" s="600" t="inlineStr">
         <is>
@@ -46042,7 +46048,11 @@
         <v/>
       </c>
       <c r="R48" s="1103" t="n"/>
-      <c r="S48" s="1106" t="n"/>
+      <c r="S48" s="1104" t="inlineStr">
+        <is>
+          <t>[⚠️ 이번 달 7번 영수증과 중복 (증빙/주문번호: 26517000000466701406)]</t>
+        </is>
+      </c>
       <c r="T48" s="1097" t="n"/>
       <c r="U48" s="988" t="n"/>
       <c r="V48" s="988" t="n"/>
@@ -46063,12 +46073,12 @@
       </c>
       <c r="D49" s="1098" t="inlineStr">
         <is>
-          <t>26327000001119045774</t>
+          <t>26957000000165619116</t>
         </is>
       </c>
       <c r="E49" s="306" t="inlineStr">
         <is>
-          <t>출장비</t>
+          <t>교통비</t>
         </is>
       </c>
       <c r="F49" s="598" t="inlineStr">
@@ -46077,19 +46087,23 @@
         </is>
       </c>
       <c r="G49" s="599" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H49" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
-        </is>
-      </c>
-      <c r="I49" s="599" t="n"/>
+          <t>여비교통비</t>
+        </is>
+      </c>
+      <c r="I49" s="599" t="inlineStr">
+        <is>
+          <t>해외</t>
+        </is>
+      </c>
       <c r="J49" s="601" t="n"/>
       <c r="K49" s="601" t="n"/>
       <c r="L49" s="601" t="n"/>
       <c r="M49" s="1099" t="n">
-        <v>40</v>
+        <v>589.9</v>
       </c>
       <c r="N49" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46108,7 +46122,11 @@
         <v/>
       </c>
       <c r="R49" s="1103" t="n"/>
-      <c r="S49" s="1106" t="n"/>
+      <c r="S49" s="1104" t="inlineStr">
+        <is>
+          <t>[⚠️ 이번 달 8번 영수증과 중복 (증빙/주문번호: 26957000000165619116)]</t>
+        </is>
+      </c>
       <c r="T49" s="1097" t="n"/>
       <c r="U49" s="988" t="n"/>
       <c r="V49" s="988" t="n"/>
@@ -46129,12 +46147,12 @@
       </c>
       <c r="D50" s="1098" t="inlineStr">
         <is>
-          <t>26327000001122217547</t>
+          <t>26447000001222315056</t>
         </is>
       </c>
       <c r="E50" s="306" t="inlineStr">
         <is>
-          <t>항공권</t>
+          <t>교통비</t>
         </is>
       </c>
       <c r="F50" s="598" t="inlineStr">
@@ -46143,7 +46161,7 @@
         </is>
       </c>
       <c r="G50" s="599" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H50" s="600" t="inlineStr">
         <is>
@@ -46159,7 +46177,7 @@
       <c r="K50" s="601" t="n"/>
       <c r="L50" s="601" t="n"/>
       <c r="M50" s="1099" t="n">
-        <v>1073</v>
+        <v>887.8</v>
       </c>
       <c r="N50" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46178,7 +46196,7 @@
         <v/>
       </c>
       <c r="R50" s="1103" t="n"/>
-      <c r="S50" s="1106" t="n"/>
+      <c r="S50" s="1105" t="n"/>
       <c r="T50" s="1097" t="n"/>
       <c r="U50" s="988" t="n"/>
       <c r="V50" s="988" t="n"/>
@@ -46199,12 +46217,12 @@
       </c>
       <c r="D51" s="1098" t="inlineStr">
         <is>
-          <t>26442000006669091216</t>
+          <t>26127000000304975197</t>
         </is>
       </c>
       <c r="E51" s="306" t="inlineStr">
         <is>
-          <t>숙박비</t>
+          <t>교통비</t>
         </is>
       </c>
       <c r="F51" s="598" t="inlineStr">
@@ -46213,7 +46231,7 @@
         </is>
       </c>
       <c r="G51" s="599" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H51" s="600" t="inlineStr">
         <is>
@@ -46229,7 +46247,7 @@
       <c r="K51" s="601" t="n"/>
       <c r="L51" s="601" t="n"/>
       <c r="M51" s="1099" t="n">
-        <v>1359</v>
+        <v>81.2</v>
       </c>
       <c r="N51" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46248,7 +46266,7 @@
         <v/>
       </c>
       <c r="R51" s="1103" t="n"/>
-      <c r="S51" s="1106" t="n"/>
+      <c r="S51" s="1105" t="n"/>
       <c r="T51" s="1097" t="n"/>
       <c r="U51" s="988" t="n"/>
       <c r="V51" s="988" t="n"/>
@@ -46269,12 +46287,12 @@
       </c>
       <c r="D52" s="1098" t="inlineStr">
         <is>
-          <t>26127000000304975197</t>
+          <t>45212619</t>
         </is>
       </c>
       <c r="E52" s="306" t="inlineStr">
         <is>
-          <t>교통비</t>
+          <t>화물운송료</t>
         </is>
       </c>
       <c r="F52" s="598" t="inlineStr">
@@ -46283,23 +46301,23 @@
         </is>
       </c>
       <c r="G52" s="599" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H52" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>해외지사비</t>
         </is>
       </c>
       <c r="I52" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J52" s="601" t="n"/>
       <c r="K52" s="601" t="n"/>
       <c r="L52" s="601" t="n"/>
       <c r="M52" s="1099" t="n">
-        <v>81.2</v>
+        <v>132.36</v>
       </c>
       <c r="N52" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46318,7 +46336,7 @@
         <v/>
       </c>
       <c r="R52" s="1103" t="n"/>
-      <c r="S52" s="1106" t="n"/>
+      <c r="S52" s="1105" t="n"/>
       <c r="T52" s="1097" t="n"/>
       <c r="U52" s="988" t="n"/>
       <c r="V52" s="988" t="n"/>
@@ -46339,12 +46357,12 @@
       </c>
       <c r="D53" s="1098" t="inlineStr">
         <is>
-          <t>26957000000150278611</t>
+          <t>26957000000162960397</t>
         </is>
       </c>
       <c r="E53" s="306" t="inlineStr">
         <is>
-          <t>택배비</t>
+          <t>통신비</t>
         </is>
       </c>
       <c r="F53" s="598" t="inlineStr">
@@ -46353,11 +46371,11 @@
         </is>
       </c>
       <c r="G53" s="599" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H53" s="600" t="inlineStr">
         <is>
-          <t>해외지사비</t>
+          <t>통신비</t>
         </is>
       </c>
       <c r="I53" s="599" t="inlineStr">
@@ -46369,7 +46387,7 @@
       <c r="K53" s="601" t="n"/>
       <c r="L53" s="601" t="n"/>
       <c r="M53" s="1099" t="n">
-        <v>378</v>
+        <v>300</v>
       </c>
       <c r="N53" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46388,7 +46406,11 @@
         <v/>
       </c>
       <c r="R53" s="1103" t="n"/>
-      <c r="S53" s="1106" t="n"/>
+      <c r="S53" s="1106" t="inlineStr">
+        <is>
+          <t>✅ 통신비 - 파표 회사코드 X</t>
+        </is>
+      </c>
       <c r="T53" s="1097" t="n"/>
       <c r="U53" s="988" t="n"/>
       <c r="V53" s="988" t="n"/>
@@ -46409,12 +46431,12 @@
       </c>
       <c r="D54" s="1098" t="inlineStr">
         <is>
-          <t>26957000000162960397</t>
+          <t>26327000001122217547</t>
         </is>
       </c>
       <c r="E54" s="306" t="inlineStr">
         <is>
-          <t>통신비</t>
+          <t>항공권</t>
         </is>
       </c>
       <c r="F54" s="598" t="inlineStr">
@@ -46423,23 +46445,23 @@
         </is>
       </c>
       <c r="G54" s="599" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H54" s="600" t="inlineStr">
         <is>
-          <t>통신비</t>
+          <t>여비교통비</t>
         </is>
       </c>
       <c r="I54" s="599" t="inlineStr">
         <is>
-          <t>기타</t>
+          <t>해외</t>
         </is>
       </c>
       <c r="J54" s="601" t="n"/>
       <c r="K54" s="601" t="n"/>
       <c r="L54" s="601" t="n"/>
       <c r="M54" s="1099" t="n">
-        <v>300</v>
+        <v>1073</v>
       </c>
       <c r="N54" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46458,11 +46480,7 @@
         <v/>
       </c>
       <c r="R54" s="1103" t="n"/>
-      <c r="S54" s="1104" t="inlineStr">
-        <is>
-          <t>✅ 통신비 - 파표 회사코드 X</t>
-        </is>
-      </c>
+      <c r="S54" s="1105" t="n"/>
       <c r="T54" s="1097" t="n"/>
       <c r="U54" s="988" t="n"/>
       <c r="V54" s="988" t="n"/>
@@ -46471,12 +46489,24 @@
     </row>
     <row r="55" ht="12" customFormat="1" customHeight="1" s="1089">
       <c r="A55" s="537" t="n"/>
-      <c r="B55" s="1098" t="n"/>
-      <c r="C55" s="1098" t="n"/>
-      <c r="D55" s="1098" t="inlineStr"/>
+      <c r="B55" s="1098" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C55" s="1098" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="D55" s="1098" t="inlineStr">
+        <is>
+          <t>26327000001119045774</t>
+        </is>
+      </c>
       <c r="E55" s="306" t="inlineStr">
         <is>
-          <t>톨비/주차비</t>
+          <t>출장비</t>
         </is>
       </c>
       <c r="F55" s="598" t="inlineStr">
@@ -46485,23 +46515,19 @@
         </is>
       </c>
       <c r="G55" s="599" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H55" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
-        </is>
-      </c>
-      <c r="I55" s="599" t="inlineStr">
-        <is>
-          <t>해외</t>
-        </is>
-      </c>
+          <t>해외지사비</t>
+        </is>
+      </c>
+      <c r="I55" s="599" t="n"/>
       <c r="J55" s="601" t="n"/>
       <c r="K55" s="601" t="n"/>
       <c r="L55" s="601" t="n"/>
       <c r="M55" s="1099" t="n">
-        <v>149</v>
+        <v>40</v>
       </c>
       <c r="N55" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46520,11 +46546,7 @@
         <v/>
       </c>
       <c r="R55" s="1103" t="n"/>
-      <c r="S55" s="1105" t="inlineStr">
-        <is>
-          <t>파표 외 영수증</t>
-        </is>
-      </c>
+      <c r="S55" s="1105" t="n"/>
       <c r="T55" s="1097" t="n"/>
       <c r="U55" s="988" t="n"/>
       <c r="V55" s="988" t="n"/>
@@ -46533,12 +46555,24 @@
     </row>
     <row r="56" ht="12" customFormat="1" customHeight="1" s="1089">
       <c r="A56" s="537" t="n"/>
-      <c r="B56" s="1098" t="n"/>
-      <c r="C56" s="1098" t="n"/>
-      <c r="D56" s="1098" t="inlineStr"/>
+      <c r="B56" s="1098" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C56" s="1098" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="D56" s="1098" t="inlineStr">
+        <is>
+          <t>26327000001122217548</t>
+        </is>
+      </c>
       <c r="E56" s="306" t="inlineStr">
         <is>
-          <t>톨비/주차비</t>
+          <t>항공권</t>
         </is>
       </c>
       <c r="F56" s="598" t="inlineStr">
@@ -46547,7 +46581,7 @@
         </is>
       </c>
       <c r="G56" s="599" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H56" s="600" t="inlineStr">
         <is>
@@ -46563,7 +46597,7 @@
       <c r="K56" s="601" t="n"/>
       <c r="L56" s="601" t="n"/>
       <c r="M56" s="1099" t="n">
-        <v>149</v>
+        <v>63</v>
       </c>
       <c r="N56" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46582,11 +46616,7 @@
         <v/>
       </c>
       <c r="R56" s="1103" t="n"/>
-      <c r="S56" s="1105" t="inlineStr">
-        <is>
-          <t>파표 외 영수증</t>
-        </is>
-      </c>
+      <c r="S56" s="1105" t="n"/>
       <c r="T56" s="1097" t="n"/>
       <c r="U56" s="988" t="n"/>
       <c r="V56" s="988" t="n"/>
@@ -46595,33 +46625,49 @@
     </row>
     <row r="57" ht="12" customFormat="1" customHeight="1" s="1089">
       <c r="A57" s="537" t="n"/>
-      <c r="B57" s="1098" t="n"/>
-      <c r="C57" s="1098" t="n"/>
-      <c r="D57" s="1098" t="inlineStr"/>
-      <c r="E57" s="306" t="n"/>
+      <c r="B57" s="1098" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="C57" s="1098" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="D57" s="1098" t="inlineStr">
+        <is>
+          <t>26957000000150278611</t>
+        </is>
+      </c>
+      <c r="E57" s="306" t="inlineStr">
+        <is>
+          <t>택배비</t>
+        </is>
+      </c>
       <c r="F57" s="598" t="inlineStr">
         <is>
           <t>Lin Wei Jian</t>
         </is>
       </c>
       <c r="G57" s="599" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H57" s="600" t="inlineStr">
         <is>
-          <t>여비교통비</t>
+          <t>해외지사비</t>
         </is>
       </c>
       <c r="I57" s="599" t="inlineStr">
         <is>
-          <t>해외</t>
+          <t>기타</t>
         </is>
       </c>
       <c r="J57" s="601" t="n"/>
       <c r="K57" s="601" t="n"/>
       <c r="L57" s="601" t="n"/>
       <c r="M57" s="1099" t="n">
-        <v>102.7</v>
+        <v>378</v>
       </c>
       <c r="N57" s="1100">
         <f>'통장내역(환율표)'!D94</f>
@@ -46640,11 +46686,7 @@
         <v/>
       </c>
       <c r="R57" s="1103" t="n"/>
-      <c r="S57" s="1105" t="inlineStr">
-        <is>
-          <t>파표 외 영수증</t>
-        </is>
-      </c>
+      <c r="S57" s="1105" t="n"/>
       <c r="T57" s="1097" t="n"/>
       <c r="U57" s="988" t="n"/>
       <c r="V57" s="988" t="n"/>
@@ -46655,22 +46697,54 @@
       <c r="A58" s="537" t="n"/>
       <c r="B58" s="1098" t="n"/>
       <c r="C58" s="1098" t="n"/>
-      <c r="D58" s="1098" t="n"/>
+      <c r="D58" s="1098" t="inlineStr"/>
       <c r="E58" s="306" t="n"/>
-      <c r="F58" s="598" t="n"/>
-      <c r="G58" s="599" t="n"/>
-      <c r="H58" s="600" t="n"/>
-      <c r="I58" s="599" t="n"/>
+      <c r="F58" s="598" t="inlineStr">
+        <is>
+          <t>Lin Wei Jian</t>
+        </is>
+      </c>
+      <c r="G58" s="599" t="n">
+        <v>37</v>
+      </c>
+      <c r="H58" s="600" t="inlineStr">
+        <is>
+          <t>여비교통비</t>
+        </is>
+      </c>
+      <c r="I58" s="599" t="inlineStr">
+        <is>
+          <t>해외</t>
+        </is>
+      </c>
       <c r="J58" s="601" t="n"/>
       <c r="K58" s="601" t="n"/>
       <c r="L58" s="601" t="n"/>
-      <c r="M58" s="1099" t="n"/>
-      <c r="N58" s="1100" t="n"/>
-      <c r="O58" s="1101" t="n"/>
-      <c r="P58" s="1102" t="n"/>
-      <c r="Q58" s="1102" t="n"/>
+      <c r="M58" s="1099" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="N58" s="1100">
+        <f>'통장내역(환율표)'!D94</f>
+        <v/>
+      </c>
+      <c r="O58" s="1101">
+        <f>M58/N58</f>
+        <v/>
+      </c>
+      <c r="P58" s="1102">
+        <f>P57+J58-M58</f>
+        <v/>
+      </c>
+      <c r="Q58" s="1102">
+        <f>Q57+L58-O58</f>
+        <v/>
+      </c>
       <c r="R58" s="1103" t="n"/>
-      <c r="S58" s="1106" t="n"/>
+      <c r="S58" s="1104" t="inlineStr">
+        <is>
+          <t>파표 외 영수증</t>
+        </is>
+      </c>
       <c r="T58" s="1097" t="n"/>
       <c r="U58" s="988" t="n"/>
       <c r="V58" s="988" t="n"/>
@@ -46681,22 +46755,58 @@
       <c r="A59" s="537" t="n"/>
       <c r="B59" s="1098" t="n"/>
       <c r="C59" s="1098" t="n"/>
-      <c r="D59" s="1098" t="n"/>
-      <c r="E59" s="306" t="n"/>
-      <c r="F59" s="598" t="n"/>
-      <c r="G59" s="599" t="n"/>
-      <c r="H59" s="600" t="n"/>
-      <c r="I59" s="599" t="n"/>
+      <c r="D59" s="1098" t="inlineStr"/>
+      <c r="E59" s="306" t="inlineStr">
+        <is>
+          <t>톨비/주차비</t>
+        </is>
+      </c>
+      <c r="F59" s="598" t="inlineStr">
+        <is>
+          <t>Lin Wei Jian</t>
+        </is>
+      </c>
+      <c r="G59" s="599" t="n">
+        <v>38</v>
+      </c>
+      <c r="H59" s="600" t="inlineStr">
+        <is>
+          <t>여비교통비</t>
+        </is>
+      </c>
+      <c r="I59" s="599" t="inlineStr">
+        <is>
+          <t>해외</t>
+        </is>
+      </c>
       <c r="J59" s="601" t="n"/>
       <c r="K59" s="601" t="n"/>
       <c r="L59" s="601" t="n"/>
-      <c r="M59" s="1099" t="n"/>
-      <c r="N59" s="1100" t="n"/>
-      <c r="O59" s="1101" t="n"/>
-      <c r="P59" s="1102" t="n"/>
-      <c r="Q59" s="1102" t="n"/>
+      <c r="M59" s="1099" t="n">
+        <v>149</v>
+      </c>
+      <c r="N59" s="1100">
+        <f>'통장내역(환율표)'!D94</f>
+        <v/>
+      </c>
+      <c r="O59" s="1101">
+        <f>M59/N59</f>
+        <v/>
+      </c>
+      <c r="P59" s="1102">
+        <f>P58+J59-M59</f>
+        <v/>
+      </c>
+      <c r="Q59" s="1102">
+        <f>Q58+L59-O59</f>
+        <v/>
+      </c>
       <c r="R59" s="1103" t="n"/>
-      <c r="S59" s="1106" t="n"/>
+      <c r="S59" s="1104" t="inlineStr">
+        <is>
+          <t>파표 외 영수증</t>
+        </is>
+      </c>
       <c r="T59" s="1097" t="n"/>
       <c r="U59" s="988" t="n"/>
       <c r="V59" s="988" t="n"/>
@@ -46707,22 +46817,58 @@
       <c r="A60" s="537" t="n"/>
       <c r="B60" s="1098" t="n"/>
       <c r="C60" s="1098" t="n"/>
-      <c r="D60" s="1098" t="n"/>
-      <c r="E60" s="306" t="n"/>
-      <c r="F60" s="598" t="n"/>
-      <c r="G60" s="599" t="n"/>
-      <c r="H60" s="600" t="n"/>
-      <c r="I60" s="599" t="n"/>
+      <c r="D60" s="1098" t="inlineStr"/>
+      <c r="E60" s="306" t="inlineStr">
+        <is>
+          <t>톨비/주차비</t>
+        </is>
+      </c>
+      <c r="F60" s="598" t="inlineStr">
+        <is>
+          <t>Lin Wei Jian</t>
+        </is>
+      </c>
+      <c r="G60" s="599" t="n">
+        <v>39</v>
+      </c>
+      <c r="H60" s="600" t="inlineStr">
+        <is>
+          <t>여비교통비</t>
+        </is>
+      </c>
+      <c r="I60" s="599" t="inlineStr">
+        <is>
+          <t>해외</t>
+        </is>
+      </c>
       <c r="J60" s="601" t="n"/>
       <c r="K60" s="601" t="n"/>
       <c r="L60" s="601" t="n"/>
-      <c r="M60" s="1099" t="n"/>
-      <c r="N60" s="1100" t="n"/>
-      <c r="O60" s="1101" t="n"/>
-      <c r="P60" s="1102" t="n"/>
-      <c r="Q60" s="1102" t="n"/>
+      <c r="M60" s="1099" t="n">
+        <v>149</v>
+      </c>
+      <c r="N60" s="1100">
+        <f>'통장내역(환율표)'!D94</f>
+        <v/>
+      </c>
+      <c r="O60" s="1101">
+        <f>M60/N60</f>
+        <v/>
+      </c>
+      <c r="P60" s="1102">
+        <f>P59+J60-M60</f>
+        <v/>
+      </c>
+      <c r="Q60" s="1102">
+        <f>Q59+L60-O60</f>
+        <v/>
+      </c>
       <c r="R60" s="1103" t="n"/>
-      <c r="S60" s="1106" t="n"/>
+      <c r="S60" s="1104" t="inlineStr">
+        <is>
+          <t>파표 외 영수증</t>
+        </is>
+      </c>
       <c r="T60" s="1097" t="n"/>
       <c r="U60" s="988" t="n"/>
       <c r="V60" s="988" t="n"/>
@@ -46748,7 +46894,7 @@
       <c r="P61" s="1102" t="n"/>
       <c r="Q61" s="1102" t="n"/>
       <c r="R61" s="1103" t="n"/>
-      <c r="S61" s="1106" t="n"/>
+      <c r="S61" s="1105" t="n"/>
       <c r="T61" s="1097" t="n"/>
       <c r="U61" s="988" t="n"/>
       <c r="V61" s="988" t="n"/>
@@ -46774,7 +46920,7 @@
       <c r="P62" s="1102" t="n"/>
       <c r="Q62" s="1102" t="n"/>
       <c r="R62" s="1103" t="n"/>
-      <c r="S62" s="1106" t="n"/>
+      <c r="S62" s="1105" t="n"/>
       <c r="T62" s="1097" t="n"/>
       <c r="U62" s="988" t="n"/>
       <c r="V62" s="988" t="n"/>
@@ -46800,7 +46946,7 @@
       <c r="P63" s="1102" t="n"/>
       <c r="Q63" s="1102" t="n"/>
       <c r="R63" s="1103" t="n"/>
-      <c r="S63" s="1106" t="n"/>
+      <c r="S63" s="1105" t="n"/>
       <c r="T63" s="1097" t="n"/>
       <c r="U63" s="988" t="n"/>
       <c r="V63" s="988" t="n"/>
@@ -46826,7 +46972,7 @@
       <c r="P64" s="1102" t="n"/>
       <c r="Q64" s="1102" t="n"/>
       <c r="R64" s="1103" t="n"/>
-      <c r="S64" s="1106" t="n"/>
+      <c r="S64" s="1105" t="n"/>
       <c r="T64" s="1097" t="n"/>
       <c r="U64" s="988" t="n"/>
       <c r="V64" s="988" t="n"/>
@@ -46852,7 +46998,7 @@
       <c r="P65" s="1102" t="n"/>
       <c r="Q65" s="1102" t="n"/>
       <c r="R65" s="1103" t="n"/>
-      <c r="S65" s="1106" t="n"/>
+      <c r="S65" s="1105" t="n"/>
       <c r="T65" s="1097" t="n"/>
       <c r="U65" s="988" t="n"/>
       <c r="V65" s="988" t="n"/>
@@ -46878,7 +47024,7 @@
       <c r="P66" s="1102" t="n"/>
       <c r="Q66" s="1102" t="n"/>
       <c r="R66" s="1103" t="n"/>
-      <c r="S66" s="1106" t="n"/>
+      <c r="S66" s="1105" t="n"/>
       <c r="T66" s="1097" t="n"/>
       <c r="U66" s="988" t="n"/>
       <c r="V66" s="988" t="n"/>
@@ -46904,7 +47050,7 @@
       <c r="P67" s="1102" t="n"/>
       <c r="Q67" s="1102" t="n"/>
       <c r="R67" s="1103" t="n"/>
-      <c r="S67" s="1106" t="n"/>
+      <c r="S67" s="1105" t="n"/>
       <c r="T67" s="1097" t="n"/>
       <c r="U67" s="988" t="n"/>
       <c r="V67" s="988" t="n"/>
@@ -46930,7 +47076,7 @@
       <c r="P68" s="1102" t="n"/>
       <c r="Q68" s="1102" t="n"/>
       <c r="R68" s="1103" t="n"/>
-      <c r="S68" s="1106" t="n"/>
+      <c r="S68" s="1105" t="n"/>
       <c r="T68" s="1097" t="n"/>
       <c r="U68" s="988" t="n"/>
       <c r="V68" s="988" t="n"/>
@@ -46956,7 +47102,7 @@
       <c r="P69" s="1102" t="n"/>
       <c r="Q69" s="1102" t="n"/>
       <c r="R69" s="1103" t="n"/>
-      <c r="S69" s="1106" t="n"/>
+      <c r="S69" s="1105" t="n"/>
       <c r="T69" s="1097" t="n"/>
       <c r="U69" s="988" t="n"/>
       <c r="V69" s="988" t="n"/>
@@ -46982,7 +47128,7 @@
       <c r="P70" s="1102" t="n"/>
       <c r="Q70" s="1102" t="n"/>
       <c r="R70" s="1103" t="n"/>
-      <c r="S70" s="1106" t="n"/>
+      <c r="S70" s="1105" t="n"/>
       <c r="T70" s="1097" t="n"/>
       <c r="U70" s="988" t="n"/>
       <c r="V70" s="988" t="n"/>
@@ -47008,7 +47154,7 @@
       <c r="P71" s="1102" t="n"/>
       <c r="Q71" s="1102" t="n"/>
       <c r="R71" s="1103" t="n"/>
-      <c r="S71" s="1106" t="n"/>
+      <c r="S71" s="1105" t="n"/>
       <c r="T71" s="1097" t="n"/>
       <c r="U71" s="988" t="n"/>
       <c r="V71" s="988" t="n"/>
@@ -47034,7 +47180,7 @@
       <c r="P72" s="1102" t="n"/>
       <c r="Q72" s="1102" t="n"/>
       <c r="R72" s="1103" t="n"/>
-      <c r="S72" s="1106" t="n"/>
+      <c r="S72" s="1105" t="n"/>
       <c r="T72" s="1097" t="n"/>
       <c r="U72" s="988" t="n"/>
       <c r="V72" s="988" t="n"/>
@@ -47060,7 +47206,7 @@
       <c r="P73" s="1102" t="n"/>
       <c r="Q73" s="1102" t="n"/>
       <c r="R73" s="1103" t="n"/>
-      <c r="S73" s="1106" t="n"/>
+      <c r="S73" s="1105" t="n"/>
       <c r="T73" s="1097" t="n"/>
       <c r="U73" s="988" t="n"/>
       <c r="V73" s="988" t="n"/>
@@ -47086,7 +47232,7 @@
       <c r="P74" s="1102" t="n"/>
       <c r="Q74" s="1102" t="n"/>
       <c r="R74" s="1103" t="n"/>
-      <c r="S74" s="1106" t="n"/>
+      <c r="S74" s="1105" t="n"/>
       <c r="T74" s="1097" t="n"/>
       <c r="U74" s="988" t="n"/>
       <c r="V74" s="988" t="n"/>
@@ -47112,7 +47258,7 @@
       <c r="P75" s="1102" t="n"/>
       <c r="Q75" s="1102" t="n"/>
       <c r="R75" s="1103" t="n"/>
-      <c r="S75" s="1106" t="n"/>
+      <c r="S75" s="1105" t="n"/>
       <c r="T75" s="1097" t="n"/>
       <c r="U75" s="988" t="n"/>
       <c r="V75" s="988" t="n"/>
@@ -47138,7 +47284,7 @@
       <c r="P76" s="1102" t="n"/>
       <c r="Q76" s="1102" t="n"/>
       <c r="R76" s="1103" t="n"/>
-      <c r="S76" s="1106" t="n"/>
+      <c r="S76" s="1105" t="n"/>
       <c r="T76" s="1097" t="n"/>
       <c r="U76" s="988" t="n"/>
       <c r="V76" s="988" t="n"/>
@@ -47164,7 +47310,7 @@
       <c r="P77" s="1102" t="n"/>
       <c r="Q77" s="1102" t="n"/>
       <c r="R77" s="1103" t="n"/>
-      <c r="S77" s="1106" t="n"/>
+      <c r="S77" s="1105" t="n"/>
       <c r="T77" s="1097" t="n"/>
       <c r="U77" s="988" t="n"/>
       <c r="V77" s="988" t="n"/>
@@ -47190,7 +47336,7 @@
       <c r="P78" s="1102" t="n"/>
       <c r="Q78" s="1102" t="n"/>
       <c r="R78" s="1103" t="n"/>
-      <c r="S78" s="1106" t="n"/>
+      <c r="S78" s="1105" t="n"/>
       <c r="T78" s="1097" t="n"/>
       <c r="U78" s="988" t="n"/>
       <c r="V78" s="988" t="n"/>
@@ -47216,7 +47362,7 @@
       <c r="P79" s="1102" t="n"/>
       <c r="Q79" s="1102" t="n"/>
       <c r="R79" s="1103" t="n"/>
-      <c r="S79" s="1106" t="n"/>
+      <c r="S79" s="1105" t="n"/>
       <c r="T79" s="1097" t="n"/>
       <c r="U79" s="988" t="n"/>
       <c r="V79" s="988" t="n"/>
@@ -47242,7 +47388,7 @@
       <c r="P80" s="1102" t="n"/>
       <c r="Q80" s="1102" t="n"/>
       <c r="R80" s="1103" t="n"/>
-      <c r="S80" s="1106" t="n"/>
+      <c r="S80" s="1105" t="n"/>
       <c r="T80" s="1097" t="n"/>
       <c r="U80" s="988" t="n"/>
       <c r="V80" s="988" t="n"/>
@@ -47268,7 +47414,7 @@
       <c r="P81" s="1102" t="n"/>
       <c r="Q81" s="1102" t="n"/>
       <c r="R81" s="1103" t="n"/>
-      <c r="S81" s="1106" t="n"/>
+      <c r="S81" s="1105" t="n"/>
       <c r="T81" s="1097" t="n"/>
       <c r="U81" s="988" t="n"/>
       <c r="V81" s="988" t="n"/>
@@ -47294,7 +47440,7 @@
       <c r="P82" s="1102" t="n"/>
       <c r="Q82" s="1102" t="n"/>
       <c r="R82" s="1103" t="n"/>
-      <c r="S82" s="1106" t="n"/>
+      <c r="S82" s="1105" t="n"/>
       <c r="T82" s="1097" t="n"/>
       <c r="U82" s="988" t="n"/>
       <c r="V82" s="988" t="n"/>
@@ -47320,7 +47466,7 @@
       <c r="P83" s="1102" t="n"/>
       <c r="Q83" s="1102" t="n"/>
       <c r="R83" s="1103" t="n"/>
-      <c r="S83" s="1106" t="n"/>
+      <c r="S83" s="1105" t="n"/>
       <c r="T83" s="1097" t="n"/>
       <c r="U83" s="988" t="n"/>
       <c r="V83" s="988" t="n"/>
@@ -47346,7 +47492,7 @@
       <c r="P84" s="1102" t="n"/>
       <c r="Q84" s="1102" t="n"/>
       <c r="R84" s="1103" t="n"/>
-      <c r="S84" s="1106" t="n"/>
+      <c r="S84" s="1105" t="n"/>
       <c r="T84" s="1097" t="n"/>
       <c r="U84" s="988" t="n"/>
       <c r="V84" s="988" t="n"/>
@@ -47372,7 +47518,7 @@
       <c r="P85" s="1102" t="n"/>
       <c r="Q85" s="1102" t="n"/>
       <c r="R85" s="1103" t="n"/>
-      <c r="S85" s="1106" t="n"/>
+      <c r="S85" s="1105" t="n"/>
       <c r="T85" s="1097" t="n"/>
       <c r="U85" s="988" t="n"/>
       <c r="V85" s="988" t="n"/>
@@ -47398,7 +47544,7 @@
       <c r="P86" s="1102" t="n"/>
       <c r="Q86" s="1102" t="n"/>
       <c r="R86" s="1103" t="n"/>
-      <c r="S86" s="1106" t="n"/>
+      <c r="S86" s="1105" t="n"/>
       <c r="T86" s="1097" t="n"/>
       <c r="U86" s="988" t="n"/>
       <c r="V86" s="988" t="n"/>
@@ -47424,7 +47570,7 @@
       <c r="P87" s="1102" t="n"/>
       <c r="Q87" s="1102" t="n"/>
       <c r="R87" s="1103" t="n"/>
-      <c r="S87" s="1106" t="n"/>
+      <c r="S87" s="1105" t="n"/>
       <c r="T87" s="1097" t="n"/>
       <c r="U87" s="988" t="n"/>
       <c r="V87" s="988" t="n"/>
@@ -47450,7 +47596,7 @@
       <c r="P88" s="1102" t="n"/>
       <c r="Q88" s="1102" t="n"/>
       <c r="R88" s="1103" t="n"/>
-      <c r="S88" s="1106" t="n"/>
+      <c r="S88" s="1105" t="n"/>
       <c r="T88" s="1097" t="n"/>
       <c r="U88" s="988" t="n"/>
       <c r="V88" s="988" t="n"/>
@@ -47476,7 +47622,7 @@
       <c r="P89" s="1102" t="n"/>
       <c r="Q89" s="1102" t="n"/>
       <c r="R89" s="1103" t="n"/>
-      <c r="S89" s="1106" t="n"/>
+      <c r="S89" s="1105" t="n"/>
       <c r="T89" s="1097" t="n"/>
       <c r="U89" s="988" t="n"/>
       <c r="V89" s="988" t="n"/>
@@ -47502,7 +47648,7 @@
       <c r="P90" s="1102" t="n"/>
       <c r="Q90" s="1102" t="n"/>
       <c r="R90" s="1103" t="n"/>
-      <c r="S90" s="1106" t="n"/>
+      <c r="S90" s="1105" t="n"/>
       <c r="T90" s="1097" t="n"/>
       <c r="U90" s="988" t="n"/>
       <c r="V90" s="988" t="n"/>
@@ -47528,7 +47674,7 @@
       <c r="P91" s="1102" t="n"/>
       <c r="Q91" s="1102" t="n"/>
       <c r="R91" s="1103" t="n"/>
-      <c r="S91" s="1106" t="n"/>
+      <c r="S91" s="1105" t="n"/>
       <c r="T91" s="1097" t="n"/>
       <c r="U91" s="988" t="n"/>
       <c r="V91" s="988" t="n"/>
@@ -47554,7 +47700,7 @@
       <c r="P92" s="1102" t="n"/>
       <c r="Q92" s="1102" t="n"/>
       <c r="R92" s="1103" t="n"/>
-      <c r="S92" s="1106" t="n"/>
+      <c r="S92" s="1105" t="n"/>
       <c r="T92" s="1097" t="n"/>
       <c r="U92" s="988" t="n"/>
       <c r="V92" s="988" t="n"/>
@@ -47580,7 +47726,7 @@
       <c r="P93" s="1102" t="n"/>
       <c r="Q93" s="1102" t="n"/>
       <c r="R93" s="1103" t="n"/>
-      <c r="S93" s="1106" t="n"/>
+      <c r="S93" s="1105" t="n"/>
       <c r="T93" s="1097" t="n"/>
       <c r="U93" s="988" t="n"/>
       <c r="V93" s="988" t="n"/>
@@ -47606,7 +47752,7 @@
       <c r="P94" s="1102" t="n"/>
       <c r="Q94" s="1102" t="n"/>
       <c r="R94" s="1103" t="n"/>
-      <c r="S94" s="1106" t="n"/>
+      <c r="S94" s="1105" t="n"/>
       <c r="T94" s="1097" t="n"/>
       <c r="U94" s="988" t="n"/>
       <c r="V94" s="988" t="n"/>
@@ -47632,7 +47778,7 @@
       <c r="P95" s="1102" t="n"/>
       <c r="Q95" s="1102" t="n"/>
       <c r="R95" s="1103" t="n"/>
-      <c r="S95" s="1106" t="n"/>
+      <c r="S95" s="1105" t="n"/>
       <c r="T95" s="1097" t="n"/>
       <c r="U95" s="988" t="n"/>
       <c r="V95" s="988" t="n"/>
@@ -47658,7 +47804,7 @@
       <c r="P96" s="1102" t="n"/>
       <c r="Q96" s="1102" t="n"/>
       <c r="R96" s="1103" t="n"/>
-      <c r="S96" s="1106" t="n"/>
+      <c r="S96" s="1105" t="n"/>
       <c r="T96" s="1097" t="n"/>
       <c r="U96" s="988" t="n"/>
       <c r="V96" s="988" t="n"/>
@@ -47684,7 +47830,7 @@
       <c r="P97" s="1102" t="n"/>
       <c r="Q97" s="1102" t="n"/>
       <c r="R97" s="1103" t="n"/>
-      <c r="S97" s="1106" t="n"/>
+      <c r="S97" s="1105" t="n"/>
       <c r="T97" s="1097" t="n"/>
       <c r="U97" s="988" t="n"/>
       <c r="V97" s="988" t="n"/>
@@ -47710,7 +47856,7 @@
       <c r="P98" s="1102" t="n"/>
       <c r="Q98" s="1102" t="n"/>
       <c r="R98" s="1103" t="n"/>
-      <c r="S98" s="1106" t="n"/>
+      <c r="S98" s="1105" t="n"/>
       <c r="T98" s="1097" t="n"/>
       <c r="U98" s="988" t="n"/>
       <c r="V98" s="988" t="n"/>
@@ -47736,7 +47882,7 @@
       <c r="P99" s="1102" t="n"/>
       <c r="Q99" s="1102" t="n"/>
       <c r="R99" s="1103" t="n"/>
-      <c r="S99" s="1106" t="n"/>
+      <c r="S99" s="1105" t="n"/>
       <c r="T99" s="1097" t="n"/>
       <c r="U99" s="988" t="n"/>
       <c r="V99" s="988" t="n"/>
@@ -47762,7 +47908,7 @@
       <c r="P100" s="1102" t="n"/>
       <c r="Q100" s="1102" t="n"/>
       <c r="R100" s="1103" t="n"/>
-      <c r="S100" s="1106" t="n"/>
+      <c r="S100" s="1105" t="n"/>
       <c r="T100" s="1097" t="n"/>
       <c r="U100" s="988" t="n"/>
       <c r="V100" s="988" t="n"/>
@@ -47788,7 +47934,7 @@
       <c r="P101" s="1102" t="n"/>
       <c r="Q101" s="1102" t="n"/>
       <c r="R101" s="1103" t="n"/>
-      <c r="S101" s="1106" t="n"/>
+      <c r="S101" s="1105" t="n"/>
       <c r="T101" s="1097" t="n"/>
       <c r="U101" s="988" t="n"/>
       <c r="V101" s="988" t="n"/>
@@ -47814,7 +47960,7 @@
       <c r="P102" s="1102" t="n"/>
       <c r="Q102" s="1102" t="n"/>
       <c r="R102" s="1103" t="n"/>
-      <c r="S102" s="1106" t="n"/>
+      <c r="S102" s="1105" t="n"/>
       <c r="T102" s="1097" t="n"/>
       <c r="U102" s="988" t="n"/>
       <c r="V102" s="988" t="n"/>
@@ -47840,7 +47986,7 @@
       <c r="P103" s="1102" t="n"/>
       <c r="Q103" s="1102" t="n"/>
       <c r="R103" s="1103" t="n"/>
-      <c r="S103" s="1106" t="n"/>
+      <c r="S103" s="1105" t="n"/>
       <c r="T103" s="1097" t="n"/>
       <c r="U103" s="988" t="n"/>
       <c r="V103" s="988" t="n"/>
@@ -47866,7 +48012,7 @@
       <c r="P104" s="1102" t="n"/>
       <c r="Q104" s="1102" t="n"/>
       <c r="R104" s="1103" t="n"/>
-      <c r="S104" s="1106" t="n"/>
+      <c r="S104" s="1105" t="n"/>
       <c r="T104" s="1097" t="n"/>
       <c r="U104" s="988" t="n"/>
       <c r="V104" s="988" t="n"/>
@@ -47892,7 +48038,7 @@
       <c r="P105" s="1102" t="n"/>
       <c r="Q105" s="1102" t="n"/>
       <c r="R105" s="1103" t="n"/>
-      <c r="S105" s="1106" t="n"/>
+      <c r="S105" s="1105" t="n"/>
       <c r="T105" s="1097" t="n"/>
       <c r="U105" s="988" t="n"/>
       <c r="V105" s="988" t="n"/>
@@ -47918,7 +48064,7 @@
       <c r="P106" s="1102" t="n"/>
       <c r="Q106" s="1102" t="n"/>
       <c r="R106" s="1103" t="n"/>
-      <c r="S106" s="1106" t="n"/>
+      <c r="S106" s="1105" t="n"/>
       <c r="T106" s="1097" t="n"/>
       <c r="U106" s="988" t="n"/>
       <c r="V106" s="988" t="n"/>
@@ -47944,7 +48090,7 @@
       <c r="P107" s="1102" t="n"/>
       <c r="Q107" s="1102" t="n"/>
       <c r="R107" s="1103" t="n"/>
-      <c r="S107" s="1106" t="n"/>
+      <c r="S107" s="1105" t="n"/>
       <c r="T107" s="1097" t="n"/>
       <c r="U107" s="988" t="n"/>
       <c r="V107" s="988" t="n"/>
@@ -47970,7 +48116,7 @@
       <c r="P108" s="1102" t="n"/>
       <c r="Q108" s="1102" t="n"/>
       <c r="R108" s="1103" t="n"/>
-      <c r="S108" s="1106" t="n"/>
+      <c r="S108" s="1105" t="n"/>
       <c r="T108" s="1097" t="n"/>
       <c r="U108" s="988" t="n"/>
       <c r="V108" s="988" t="n"/>
@@ -47996,7 +48142,7 @@
       <c r="P109" s="1102" t="n"/>
       <c r="Q109" s="1102" t="n"/>
       <c r="R109" s="1103" t="n"/>
-      <c r="S109" s="1106" t="n"/>
+      <c r="S109" s="1105" t="n"/>
       <c r="T109" s="1097" t="n"/>
       <c r="U109" s="988" t="n"/>
       <c r="V109" s="988" t="n"/>
@@ -48022,7 +48168,7 @@
       <c r="P110" s="1102" t="n"/>
       <c r="Q110" s="1102" t="n"/>
       <c r="R110" s="1103" t="n"/>
-      <c r="S110" s="1106" t="n"/>
+      <c r="S110" s="1105" t="n"/>
       <c r="T110" s="1097" t="n"/>
       <c r="U110" s="988" t="n"/>
       <c r="V110" s="988" t="n"/>
@@ -48048,7 +48194,7 @@
       <c r="P111" s="1102" t="n"/>
       <c r="Q111" s="1102" t="n"/>
       <c r="R111" s="1103" t="n"/>
-      <c r="S111" s="1106" t="n"/>
+      <c r="S111" s="1105" t="n"/>
       <c r="T111" s="1097" t="n"/>
       <c r="U111" s="988" t="n"/>
       <c r="V111" s="988" t="n"/>
@@ -48074,7 +48220,7 @@
       <c r="P112" s="1102" t="n"/>
       <c r="Q112" s="1102" t="n"/>
       <c r="R112" s="1103" t="n"/>
-      <c r="S112" s="1106" t="n"/>
+      <c r="S112" s="1105" t="n"/>
       <c r="T112" s="1097" t="n"/>
       <c r="U112" s="988" t="n"/>
       <c r="V112" s="988" t="n"/>
@@ -48100,7 +48246,7 @@
       <c r="P113" s="1102" t="n"/>
       <c r="Q113" s="1102" t="n"/>
       <c r="R113" s="1103" t="n"/>
-      <c r="S113" s="1106" t="n"/>
+      <c r="S113" s="1105" t="n"/>
       <c r="T113" s="1097" t="n"/>
       <c r="U113" s="988" t="n"/>
       <c r="V113" s="988" t="n"/>
@@ -48126,7 +48272,7 @@
       <c r="P114" s="1102" t="n"/>
       <c r="Q114" s="1102" t="n"/>
       <c r="R114" s="1103" t="n"/>
-      <c r="S114" s="1106" t="n"/>
+      <c r="S114" s="1105" t="n"/>
       <c r="T114" s="1097" t="n"/>
       <c r="U114" s="988" t="n"/>
       <c r="V114" s="988" t="n"/>
@@ -48152,7 +48298,7 @@
       <c r="P115" s="1102" t="n"/>
       <c r="Q115" s="1102" t="n"/>
       <c r="R115" s="1103" t="n"/>
-      <c r="S115" s="1106" t="n"/>
+      <c r="S115" s="1105" t="n"/>
       <c r="T115" s="1097" t="n"/>
       <c r="U115" s="988" t="n"/>
       <c r="V115" s="988" t="n"/>
@@ -48178,7 +48324,7 @@
       <c r="P116" s="1102" t="n"/>
       <c r="Q116" s="1102" t="n"/>
       <c r="R116" s="1103" t="n"/>
-      <c r="S116" s="1106" t="n"/>
+      <c r="S116" s="1105" t="n"/>
       <c r="T116" s="1097" t="n"/>
       <c r="U116" s="988" t="n"/>
       <c r="V116" s="988" t="n"/>
@@ -48204,7 +48350,7 @@
       <c r="P117" s="1102" t="n"/>
       <c r="Q117" s="1102" t="n"/>
       <c r="R117" s="1103" t="n"/>
-      <c r="S117" s="1106" t="n"/>
+      <c r="S117" s="1105" t="n"/>
       <c r="T117" s="1097" t="n"/>
       <c r="U117" s="988" t="n"/>
       <c r="V117" s="988" t="n"/>
@@ -48230,7 +48376,7 @@
       <c r="P118" s="1102" t="n"/>
       <c r="Q118" s="1102" t="n"/>
       <c r="R118" s="1103" t="n"/>
-      <c r="S118" s="1106" t="n"/>
+      <c r="S118" s="1105" t="n"/>
       <c r="T118" s="1097" t="n"/>
       <c r="U118" s="988" t="n"/>
       <c r="V118" s="988" t="n"/>
@@ -48256,7 +48402,7 @@
       <c r="P119" s="1102" t="n"/>
       <c r="Q119" s="1102" t="n"/>
       <c r="R119" s="1103" t="n"/>
-      <c r="S119" s="1106" t="n"/>
+      <c r="S119" s="1105" t="n"/>
       <c r="T119" s="1097" t="n"/>
       <c r="U119" s="988" t="n"/>
       <c r="V119" s="988" t="n"/>
@@ -48282,7 +48428,7 @@
       <c r="P120" s="1102" t="n"/>
       <c r="Q120" s="1102" t="n"/>
       <c r="R120" s="1103" t="n"/>
-      <c r="S120" s="1106" t="n"/>
+      <c r="S120" s="1105" t="n"/>
       <c r="T120" s="1097" t="n"/>
       <c r="U120" s="988" t="n"/>
       <c r="V120" s="988" t="n"/>
@@ -48308,7 +48454,7 @@
       <c r="P121" s="1102" t="n"/>
       <c r="Q121" s="1102" t="n"/>
       <c r="R121" s="1103" t="n"/>
-      <c r="S121" s="1106" t="n"/>
+      <c r="S121" s="1105" t="n"/>
       <c r="T121" s="1097" t="n"/>
       <c r="U121" s="988" t="n"/>
       <c r="V121" s="988" t="n"/>
@@ -48334,7 +48480,7 @@
       <c r="P122" s="1102" t="n"/>
       <c r="Q122" s="1102" t="n"/>
       <c r="R122" s="1103" t="n"/>
-      <c r="S122" s="1106" t="n"/>
+      <c r="S122" s="1105" t="n"/>
       <c r="T122" s="1097" t="n"/>
       <c r="U122" s="988" t="n"/>
       <c r="V122" s="988" t="n"/>
@@ -48360,7 +48506,7 @@
       <c r="P123" s="1102" t="n"/>
       <c r="Q123" s="1102" t="n"/>
       <c r="R123" s="1103" t="n"/>
-      <c r="S123" s="1106" t="n"/>
+      <c r="S123" s="1105" t="n"/>
       <c r="T123" s="1097" t="n"/>
       <c r="U123" s="988" t="n"/>
       <c r="V123" s="988" t="n"/>
@@ -48386,7 +48532,7 @@
       <c r="P124" s="1102" t="n"/>
       <c r="Q124" s="1102" t="n"/>
       <c r="R124" s="1103" t="n"/>
-      <c r="S124" s="1106" t="n"/>
+      <c r="S124" s="1105" t="n"/>
       <c r="T124" s="1097" t="n"/>
       <c r="U124" s="988" t="n"/>
       <c r="V124" s="988" t="n"/>
@@ -48412,7 +48558,7 @@
       <c r="P125" s="1102" t="n"/>
       <c r="Q125" s="1102" t="n"/>
       <c r="R125" s="1103" t="n"/>
-      <c r="S125" s="1106" t="n"/>
+      <c r="S125" s="1105" t="n"/>
       <c r="T125" s="1097" t="n"/>
       <c r="U125" s="988" t="n"/>
       <c r="V125" s="988" t="n"/>
@@ -48438,7 +48584,7 @@
       <c r="P126" s="1102" t="n"/>
       <c r="Q126" s="1102" t="n"/>
       <c r="R126" s="1103" t="n"/>
-      <c r="S126" s="1106" t="n"/>
+      <c r="S126" s="1105" t="n"/>
       <c r="T126" s="1097" t="n"/>
       <c r="U126" s="988" t="n"/>
       <c r="V126" s="988" t="n"/>
@@ -48464,7 +48610,7 @@
       <c r="P127" s="1102" t="n"/>
       <c r="Q127" s="1102" t="n"/>
       <c r="R127" s="1103" t="n"/>
-      <c r="S127" s="1106" t="n"/>
+      <c r="S127" s="1105" t="n"/>
       <c r="T127" s="1097" t="n"/>
       <c r="U127" s="988" t="n"/>
       <c r="V127" s="988" t="n"/>
@@ -48490,7 +48636,7 @@
       <c r="P128" s="1102" t="n"/>
       <c r="Q128" s="1102" t="n"/>
       <c r="R128" s="1103" t="n"/>
-      <c r="S128" s="1106" t="n"/>
+      <c r="S128" s="1105" t="n"/>
       <c r="T128" s="1097" t="n"/>
       <c r="U128" s="988" t="n"/>
       <c r="V128" s="988" t="n"/>
@@ -48516,7 +48662,7 @@
       <c r="P129" s="1102" t="n"/>
       <c r="Q129" s="1102" t="n"/>
       <c r="R129" s="1103" t="n"/>
-      <c r="S129" s="1106" t="n"/>
+      <c r="S129" s="1105" t="n"/>
       <c r="T129" s="1097" t="n"/>
       <c r="U129" s="988" t="n"/>
       <c r="V129" s="988" t="n"/>
@@ -48542,7 +48688,7 @@
       <c r="P130" s="1102" t="n"/>
       <c r="Q130" s="1102" t="n"/>
       <c r="R130" s="1103" t="n"/>
-      <c r="S130" s="1106" t="n"/>
+      <c r="S130" s="1105" t="n"/>
       <c r="T130" s="1097" t="n"/>
       <c r="U130" s="988" t="n"/>
       <c r="V130" s="988" t="n"/>
@@ -48568,7 +48714,7 @@
       <c r="P131" s="1102" t="n"/>
       <c r="Q131" s="1102" t="n"/>
       <c r="R131" s="1103" t="n"/>
-      <c r="S131" s="1106" t="n"/>
+      <c r="S131" s="1105" t="n"/>
       <c r="T131" s="1097" t="n"/>
       <c r="U131" s="988" t="n"/>
       <c r="V131" s="988" t="n"/>
@@ -48594,7 +48740,7 @@
       <c r="P132" s="1102" t="n"/>
       <c r="Q132" s="1102" t="n"/>
       <c r="R132" s="1103" t="n"/>
-      <c r="S132" s="1106" t="n"/>
+      <c r="S132" s="1105" t="n"/>
       <c r="T132" s="1097" t="n"/>
       <c r="U132" s="988" t="n"/>
       <c r="V132" s="988" t="n"/>
@@ -48620,7 +48766,7 @@
       <c r="P133" s="1102" t="n"/>
       <c r="Q133" s="1102" t="n"/>
       <c r="R133" s="1103" t="n"/>
-      <c r="S133" s="1106" t="n"/>
+      <c r="S133" s="1105" t="n"/>
       <c r="T133" s="1097" t="n"/>
       <c r="U133" s="988" t="n"/>
       <c r="V133" s="988" t="n"/>
@@ -48646,7 +48792,7 @@
       <c r="P134" s="1102" t="n"/>
       <c r="Q134" s="1102" t="n"/>
       <c r="R134" s="1103" t="n"/>
-      <c r="S134" s="1106" t="n"/>
+      <c r="S134" s="1105" t="n"/>
       <c r="T134" s="1097" t="n"/>
       <c r="U134" s="988" t="n"/>
       <c r="V134" s="988" t="n"/>
@@ -48672,7 +48818,7 @@
       <c r="P135" s="1102" t="n"/>
       <c r="Q135" s="1102" t="n"/>
       <c r="R135" s="1103" t="n"/>
-      <c r="S135" s="1106" t="n"/>
+      <c r="S135" s="1105" t="n"/>
       <c r="T135" s="1097" t="n"/>
       <c r="U135" s="988" t="n"/>
       <c r="V135" s="988" t="n"/>
@@ -48698,7 +48844,7 @@
       <c r="P136" s="1102" t="n"/>
       <c r="Q136" s="1102" t="n"/>
       <c r="R136" s="1103" t="n"/>
-      <c r="S136" s="1106" t="n"/>
+      <c r="S136" s="1105" t="n"/>
       <c r="T136" s="1097" t="n"/>
       <c r="U136" s="988" t="n"/>
       <c r="V136" s="988" t="n"/>
@@ -48724,7 +48870,7 @@
       <c r="P137" s="1102" t="n"/>
       <c r="Q137" s="1102" t="n"/>
       <c r="R137" s="1103" t="n"/>
-      <c r="S137" s="1106" t="n"/>
+      <c r="S137" s="1105" t="n"/>
       <c r="T137" s="1097" t="n"/>
       <c r="U137" s="988" t="n"/>
       <c r="V137" s="988" t="n"/>
@@ -48750,7 +48896,7 @@
       <c r="P138" s="1102" t="n"/>
       <c r="Q138" s="1102" t="n"/>
       <c r="R138" s="1103" t="n"/>
-      <c r="S138" s="1106" t="n"/>
+      <c r="S138" s="1105" t="n"/>
       <c r="T138" s="1097" t="n"/>
       <c r="U138" s="988" t="n"/>
       <c r="V138" s="988" t="n"/>
@@ -48776,7 +48922,7 @@
       <c r="P139" s="1102" t="n"/>
       <c r="Q139" s="1102" t="n"/>
       <c r="R139" s="1103" t="n"/>
-      <c r="S139" s="1106" t="n"/>
+      <c r="S139" s="1105" t="n"/>
       <c r="T139" s="1097" t="n"/>
       <c r="U139" s="988" t="n"/>
       <c r="V139" s="988" t="n"/>
@@ -48802,7 +48948,7 @@
       <c r="P140" s="1102" t="n"/>
       <c r="Q140" s="1102" t="n"/>
       <c r="R140" s="1103" t="n"/>
-      <c r="S140" s="1106" t="n"/>
+      <c r="S140" s="1105" t="n"/>
       <c r="T140" s="1097" t="n"/>
       <c r="U140" s="988" t="n"/>
       <c r="V140" s="988" t="n"/>
@@ -48828,7 +48974,7 @@
       <c r="P141" s="1102" t="n"/>
       <c r="Q141" s="1102" t="n"/>
       <c r="R141" s="1103" t="n"/>
-      <c r="S141" s="1106" t="n"/>
+      <c r="S141" s="1105" t="n"/>
       <c r="T141" s="1097" t="n"/>
       <c r="U141" s="988" t="n"/>
       <c r="V141" s="988" t="n"/>
@@ -48854,7 +49000,7 @@
       <c r="P142" s="1102" t="n"/>
       <c r="Q142" s="1102" t="n"/>
       <c r="R142" s="1103" t="n"/>
-      <c r="S142" s="1106" t="n"/>
+      <c r="S142" s="1105" t="n"/>
       <c r="T142" s="1097" t="n"/>
       <c r="U142" s="988" t="n"/>
       <c r="V142" s="988" t="n"/>
@@ -48880,7 +49026,7 @@
       <c r="P143" s="1102" t="n"/>
       <c r="Q143" s="1102" t="n"/>
       <c r="R143" s="1103" t="n"/>
-      <c r="S143" s="1106" t="n"/>
+      <c r="S143" s="1105" t="n"/>
       <c r="T143" s="1097" t="n"/>
       <c r="U143" s="988" t="n"/>
       <c r="V143" s="988" t="n"/>
@@ -48906,7 +49052,7 @@
       <c r="P144" s="1102" t="n"/>
       <c r="Q144" s="1102" t="n"/>
       <c r="R144" s="1103" t="n"/>
-      <c r="S144" s="1106" t="n"/>
+      <c r="S144" s="1105" t="n"/>
       <c r="T144" s="1097" t="n"/>
       <c r="U144" s="988" t="n"/>
       <c r="V144" s="988" t="n"/>
@@ -48932,7 +49078,7 @@
       <c r="P145" s="1102" t="n"/>
       <c r="Q145" s="1102" t="n"/>
       <c r="R145" s="1103" t="n"/>
-      <c r="S145" s="1106" t="n"/>
+      <c r="S145" s="1105" t="n"/>
       <c r="T145" s="1097" t="n"/>
       <c r="U145" s="988" t="n"/>
       <c r="V145" s="988" t="n"/>
@@ -48958,7 +49104,7 @@
       <c r="P146" s="1102" t="n"/>
       <c r="Q146" s="1102" t="n"/>
       <c r="R146" s="1103" t="n"/>
-      <c r="S146" s="1106" t="n"/>
+      <c r="S146" s="1105" t="n"/>
       <c r="T146" s="1097" t="n"/>
       <c r="U146" s="988" t="n"/>
       <c r="V146" s="988" t="n"/>
@@ -48984,7 +49130,7 @@
       <c r="P147" s="1102" t="n"/>
       <c r="Q147" s="1102" t="n"/>
       <c r="R147" s="1103" t="n"/>
-      <c r="S147" s="1106" t="n"/>
+      <c r="S147" s="1105" t="n"/>
       <c r="T147" s="1097" t="n"/>
       <c r="U147" s="988" t="n"/>
       <c r="V147" s="988" t="n"/>
@@ -49010,7 +49156,7 @@
       <c r="P148" s="1102" t="n"/>
       <c r="Q148" s="1102" t="n"/>
       <c r="R148" s="1103" t="n"/>
-      <c r="S148" s="1106" t="n"/>
+      <c r="S148" s="1105" t="n"/>
       <c r="T148" s="1097" t="n"/>
       <c r="U148" s="988" t="n"/>
       <c r="V148" s="988" t="n"/>
@@ -49036,7 +49182,7 @@
       <c r="P149" s="1102" t="n"/>
       <c r="Q149" s="1102" t="n"/>
       <c r="R149" s="1103" t="n"/>
-      <c r="S149" s="1106" t="n"/>
+      <c r="S149" s="1105" t="n"/>
       <c r="T149" s="1097" t="n"/>
       <c r="U149" s="988" t="n"/>
       <c r="V149" s="988" t="n"/>
@@ -49062,7 +49208,7 @@
       <c r="P150" s="1102" t="n"/>
       <c r="Q150" s="1102" t="n"/>
       <c r="R150" s="1103" t="n"/>
-      <c r="S150" s="1106" t="n"/>
+      <c r="S150" s="1105" t="n"/>
       <c r="T150" s="1097" t="n"/>
       <c r="U150" s="988" t="n"/>
       <c r="V150" s="988" t="n"/>
@@ -49088,7 +49234,7 @@
       <c r="P151" s="1102" t="n"/>
       <c r="Q151" s="1102" t="n"/>
       <c r="R151" s="1103" t="n"/>
-      <c r="S151" s="1106" t="n"/>
+      <c r="S151" s="1105" t="n"/>
       <c r="T151" s="1097" t="n"/>
       <c r="U151" s="988" t="n"/>
       <c r="V151" s="988" t="n"/>
@@ -49114,7 +49260,7 @@
       <c r="P152" s="1102" t="n"/>
       <c r="Q152" s="1102" t="n"/>
       <c r="R152" s="1103" t="n"/>
-      <c r="S152" s="1106" t="n"/>
+      <c r="S152" s="1105" t="n"/>
       <c r="T152" s="1097" t="n"/>
       <c r="U152" s="988" t="n"/>
       <c r="V152" s="988" t="n"/>
@@ -49140,7 +49286,7 @@
       <c r="P153" s="1102" t="n"/>
       <c r="Q153" s="1102" t="n"/>
       <c r="R153" s="1103" t="n"/>
-      <c r="S153" s="1106" t="n"/>
+      <c r="S153" s="1105" t="n"/>
       <c r="T153" s="1097" t="n"/>
       <c r="U153" s="988" t="n"/>
       <c r="V153" s="988" t="n"/>
@@ -49166,7 +49312,7 @@
       <c r="P154" s="1102" t="n"/>
       <c r="Q154" s="1102" t="n"/>
       <c r="R154" s="1103" t="n"/>
-      <c r="S154" s="1106" t="n"/>
+      <c r="S154" s="1105" t="n"/>
       <c r="T154" s="1097" t="n"/>
       <c r="U154" s="988" t="n"/>
       <c r="V154" s="988" t="n"/>
@@ -49192,7 +49338,7 @@
       <c r="P155" s="1102" t="n"/>
       <c r="Q155" s="1102" t="n"/>
       <c r="R155" s="1103" t="n"/>
-      <c r="S155" s="1106" t="n"/>
+      <c r="S155" s="1105" t="n"/>
       <c r="T155" s="1097" t="n"/>
       <c r="U155" s="988" t="n"/>
       <c r="V155" s="988" t="n"/>
@@ -49218,7 +49364,7 @@
       <c r="P156" s="1102" t="n"/>
       <c r="Q156" s="1102" t="n"/>
       <c r="R156" s="1103" t="n"/>
-      <c r="S156" s="1106" t="n"/>
+      <c r="S156" s="1105" t="n"/>
       <c r="T156" s="1097" t="n"/>
       <c r="U156" s="988" t="n"/>
       <c r="V156" s="988" t="n"/>
@@ -49244,7 +49390,7 @@
       <c r="P157" s="1102" t="n"/>
       <c r="Q157" s="1102" t="n"/>
       <c r="R157" s="1103" t="n"/>
-      <c r="S157" s="1106" t="n"/>
+      <c r="S157" s="1105" t="n"/>
       <c r="T157" s="1097" t="n"/>
       <c r="U157" s="988" t="n"/>
       <c r="V157" s="988" t="n"/>
@@ -49270,7 +49416,7 @@
       <c r="P158" s="1102" t="n"/>
       <c r="Q158" s="1102" t="n"/>
       <c r="R158" s="1103" t="n"/>
-      <c r="S158" s="1106" t="n"/>
+      <c r="S158" s="1105" t="n"/>
       <c r="T158" s="1097" t="n"/>
       <c r="U158" s="988" t="n"/>
       <c r="V158" s="988" t="n"/>
@@ -49296,7 +49442,7 @@
       <c r="P159" s="1102" t="n"/>
       <c r="Q159" s="1102" t="n"/>
       <c r="R159" s="1103" t="n"/>
-      <c r="S159" s="1106" t="n"/>
+      <c r="S159" s="1105" t="n"/>
       <c r="T159" s="1097" t="n"/>
       <c r="U159" s="988" t="n"/>
       <c r="V159" s="988" t="n"/>
@@ -49322,7 +49468,7 @@
       <c r="P160" s="1102" t="n"/>
       <c r="Q160" s="1102" t="n"/>
       <c r="R160" s="1103" t="n"/>
-      <c r="S160" s="1106" t="n"/>
+      <c r="S160" s="1105" t="n"/>
       <c r="T160" s="1097" t="n"/>
       <c r="U160" s="988" t="n"/>
       <c r="V160" s="988" t="n"/>
@@ -49348,7 +49494,7 @@
       <c r="P161" s="1102" t="n"/>
       <c r="Q161" s="1102" t="n"/>
       <c r="R161" s="1103" t="n"/>
-      <c r="S161" s="1106" t="n"/>
+      <c r="S161" s="1105" t="n"/>
       <c r="T161" s="1097" t="n"/>
       <c r="U161" s="988" t="n"/>
       <c r="V161" s="988" t="n"/>
@@ -49374,7 +49520,7 @@
       <c r="P162" s="1102" t="n"/>
       <c r="Q162" s="1102" t="n"/>
       <c r="R162" s="1103" t="n"/>
-      <c r="S162" s="1106" t="n"/>
+      <c r="S162" s="1105" t="n"/>
       <c r="T162" s="1097" t="n"/>
       <c r="U162" s="988" t="n"/>
       <c r="V162" s="988" t="n"/>
@@ -49400,7 +49546,7 @@
       <c r="P163" s="1102" t="n"/>
       <c r="Q163" s="1102" t="n"/>
       <c r="R163" s="1103" t="n"/>
-      <c r="S163" s="1106" t="n"/>
+      <c r="S163" s="1105" t="n"/>
       <c r="T163" s="1097" t="n"/>
       <c r="U163" s="988" t="n"/>
       <c r="V163" s="988" t="n"/>
@@ -49426,7 +49572,7 @@
       <c r="P164" s="1102" t="n"/>
       <c r="Q164" s="1102" t="n"/>
       <c r="R164" s="1103" t="n"/>
-      <c r="S164" s="1106" t="n"/>
+      <c r="S164" s="1105" t="n"/>
       <c r="T164" s="1097" t="n"/>
       <c r="U164" s="988" t="n"/>
       <c r="V164" s="988" t="n"/>
@@ -49452,7 +49598,7 @@
       <c r="P165" s="1102" t="n"/>
       <c r="Q165" s="1102" t="n"/>
       <c r="R165" s="1103" t="n"/>
-      <c r="S165" s="1106" t="n"/>
+      <c r="S165" s="1105" t="n"/>
       <c r="T165" s="1097" t="n"/>
       <c r="U165" s="988" t="n"/>
       <c r="V165" s="988" t="n"/>
@@ -49478,7 +49624,7 @@
       <c r="P166" s="1102" t="n"/>
       <c r="Q166" s="1102" t="n"/>
       <c r="R166" s="1103" t="n"/>
-      <c r="S166" s="1106" t="n"/>
+      <c r="S166" s="1105" t="n"/>
       <c r="T166" s="1097" t="n"/>
       <c r="U166" s="988" t="n"/>
       <c r="V166" s="988" t="n"/>
@@ -49504,7 +49650,7 @@
       <c r="P167" s="1102" t="n"/>
       <c r="Q167" s="1102" t="n"/>
       <c r="R167" s="1103" t="n"/>
-      <c r="S167" s="1106" t="n"/>
+      <c r="S167" s="1105" t="n"/>
       <c r="T167" s="1097" t="n"/>
       <c r="U167" s="988" t="n"/>
       <c r="V167" s="988" t="n"/>
@@ -49530,7 +49676,7 @@
       <c r="P168" s="1102" t="n"/>
       <c r="Q168" s="1102" t="n"/>
       <c r="R168" s="1103" t="n"/>
-      <c r="S168" s="1106" t="n"/>
+      <c r="S168" s="1105" t="n"/>
       <c r="T168" s="1097" t="n"/>
       <c r="U168" s="988" t="n"/>
       <c r="V168" s="988" t="n"/>
@@ -49556,7 +49702,7 @@
       <c r="P169" s="1102" t="n"/>
       <c r="Q169" s="1102" t="n"/>
       <c r="R169" s="1103" t="n"/>
-      <c r="S169" s="1106" t="n"/>
+      <c r="S169" s="1105" t="n"/>
       <c r="T169" s="1097" t="n"/>
       <c r="U169" s="988" t="n"/>
       <c r="V169" s="988" t="n"/>
@@ -49582,7 +49728,7 @@
       <c r="P170" s="1102" t="n"/>
       <c r="Q170" s="1102" t="n"/>
       <c r="R170" s="1103" t="n"/>
-      <c r="S170" s="1106" t="n"/>
+      <c r="S170" s="1105" t="n"/>
       <c r="T170" s="1097" t="n"/>
       <c r="U170" s="988" t="n"/>
       <c r="V170" s="988" t="n"/>
@@ -49608,7 +49754,7 @@
       <c r="P171" s="1102" t="n"/>
       <c r="Q171" s="1102" t="n"/>
       <c r="R171" s="1103" t="n"/>
-      <c r="S171" s="1106" t="n"/>
+      <c r="S171" s="1105" t="n"/>
       <c r="T171" s="1097" t="n"/>
       <c r="U171" s="988" t="n"/>
       <c r="V171" s="988" t="n"/>
@@ -49634,7 +49780,7 @@
       <c r="P172" s="1102" t="n"/>
       <c r="Q172" s="1102" t="n"/>
       <c r="R172" s="1103" t="n"/>
-      <c r="S172" s="1106" t="n"/>
+      <c r="S172" s="1105" t="n"/>
       <c r="T172" s="1097" t="n"/>
       <c r="U172" s="988" t="n"/>
       <c r="V172" s="988" t="n"/>
@@ -49660,7 +49806,7 @@
       <c r="P173" s="1102" t="n"/>
       <c r="Q173" s="1102" t="n"/>
       <c r="R173" s="1103" t="n"/>
-      <c r="S173" s="1106" t="n"/>
+      <c r="S173" s="1105" t="n"/>
       <c r="T173" s="1097" t="n"/>
       <c r="U173" s="988" t="n"/>
       <c r="V173" s="988" t="n"/>
@@ -49686,7 +49832,7 @@
       <c r="P174" s="1102" t="n"/>
       <c r="Q174" s="1102" t="n"/>
       <c r="R174" s="1103" t="n"/>
-      <c r="S174" s="1106" t="n"/>
+      <c r="S174" s="1105" t="n"/>
       <c r="T174" s="1097" t="n"/>
       <c r="U174" s="988" t="n"/>
       <c r="V174" s="988" t="n"/>
@@ -49712,7 +49858,7 @@
       <c r="P175" s="1102" t="n"/>
       <c r="Q175" s="1102" t="n"/>
       <c r="R175" s="1103" t="n"/>
-      <c r="S175" s="1106" t="n"/>
+      <c r="S175" s="1105" t="n"/>
       <c r="T175" s="1097" t="n"/>
       <c r="U175" s="988" t="n"/>
       <c r="V175" s="988" t="n"/>
@@ -49738,7 +49884,7 @@
       <c r="P176" s="1102" t="n"/>
       <c r="Q176" s="1102" t="n"/>
       <c r="R176" s="1103" t="n"/>
-      <c r="S176" s="1106" t="n"/>
+      <c r="S176" s="1105" t="n"/>
       <c r="T176" s="1097" t="n"/>
       <c r="U176" s="988" t="n"/>
       <c r="V176" s="988" t="n"/>
@@ -49764,7 +49910,7 @@
       <c r="P177" s="1102" t="n"/>
       <c r="Q177" s="1102" t="n"/>
       <c r="R177" s="1103" t="n"/>
-      <c r="S177" s="1106" t="n"/>
+      <c r="S177" s="1105" t="n"/>
       <c r="T177" s="1097" t="n"/>
       <c r="U177" s="988" t="n"/>
       <c r="V177" s="988" t="n"/>
@@ -49790,7 +49936,7 @@
       <c r="P178" s="1102" t="n"/>
       <c r="Q178" s="1102" t="n"/>
       <c r="R178" s="1103" t="n"/>
-      <c r="S178" s="1106" t="n"/>
+      <c r="S178" s="1105" t="n"/>
       <c r="T178" s="1097" t="n"/>
       <c r="U178" s="988" t="n"/>
       <c r="V178" s="988" t="n"/>
@@ -49816,7 +49962,7 @@
       <c r="P179" s="1102" t="n"/>
       <c r="Q179" s="1102" t="n"/>
       <c r="R179" s="1103" t="n"/>
-      <c r="S179" s="1106" t="n"/>
+      <c r="S179" s="1105" t="n"/>
       <c r="T179" s="1097" t="n"/>
       <c r="U179" s="988" t="n"/>
       <c r="V179" s="988" t="n"/>
@@ -49842,7 +49988,7 @@
       <c r="P180" s="1102" t="n"/>
       <c r="Q180" s="1102" t="n"/>
       <c r="R180" s="1103" t="n"/>
-      <c r="S180" s="1106" t="n"/>
+      <c r="S180" s="1105" t="n"/>
       <c r="T180" s="1097" t="n"/>
       <c r="U180" s="988" t="n"/>
       <c r="V180" s="988" t="n"/>
@@ -49868,7 +50014,7 @@
       <c r="P181" s="1102" t="n"/>
       <c r="Q181" s="1102" t="n"/>
       <c r="R181" s="1103" t="n"/>
-      <c r="S181" s="1106" t="n"/>
+      <c r="S181" s="1105" t="n"/>
       <c r="T181" s="1097" t="n"/>
       <c r="U181" s="988" t="n"/>
       <c r="V181" s="988" t="n"/>
@@ -49894,7 +50040,7 @@
       <c r="P182" s="1102" t="n"/>
       <c r="Q182" s="1102" t="n"/>
       <c r="R182" s="1103" t="n"/>
-      <c r="S182" s="1106" t="n"/>
+      <c r="S182" s="1105" t="n"/>
       <c r="T182" s="1097" t="n"/>
       <c r="U182" s="988" t="n"/>
       <c r="V182" s="988" t="n"/>
@@ -49920,7 +50066,7 @@
       <c r="P183" s="1102" t="n"/>
       <c r="Q183" s="1102" t="n"/>
       <c r="R183" s="1103" t="n"/>
-      <c r="S183" s="1106" t="n"/>
+      <c r="S183" s="1105" t="n"/>
       <c r="T183" s="1097" t="n"/>
       <c r="U183" s="988" t="n"/>
       <c r="V183" s="988" t="n"/>
@@ -49946,7 +50092,7 @@
       <c r="P184" s="1102" t="n"/>
       <c r="Q184" s="1102" t="n"/>
       <c r="R184" s="1103" t="n"/>
-      <c r="S184" s="1106" t="n"/>
+      <c r="S184" s="1105" t="n"/>
       <c r="T184" s="1097" t="n"/>
       <c r="U184" s="988" t="n"/>
       <c r="V184" s="988" t="n"/>
@@ -49972,7 +50118,7 @@
       <c r="P185" s="1102" t="n"/>
       <c r="Q185" s="1102" t="n"/>
       <c r="R185" s="1103" t="n"/>
-      <c r="S185" s="1106" t="n"/>
+      <c r="S185" s="1105" t="n"/>
       <c r="T185" s="1097" t="n"/>
       <c r="U185" s="988" t="n"/>
       <c r="V185" s="988" t="n"/>
@@ -49998,7 +50144,7 @@
       <c r="P186" s="1102" t="n"/>
       <c r="Q186" s="1102" t="n"/>
       <c r="R186" s="1103" t="n"/>
-      <c r="S186" s="1106" t="n"/>
+      <c r="S186" s="1105" t="n"/>
       <c r="T186" s="1097" t="n"/>
       <c r="U186" s="988" t="n"/>
       <c r="V186" s="988" t="n"/>
@@ -50024,7 +50170,7 @@
       <c r="P187" s="1102" t="n"/>
       <c r="Q187" s="1102" t="n"/>
       <c r="R187" s="1103" t="n"/>
-      <c r="S187" s="1106" t="n"/>
+      <c r="S187" s="1105" t="n"/>
       <c r="T187" s="1097" t="n"/>
       <c r="U187" s="988" t="n"/>
       <c r="V187" s="988" t="n"/>
@@ -50050,7 +50196,7 @@
       <c r="P188" s="1102" t="n"/>
       <c r="Q188" s="1102" t="n"/>
       <c r="R188" s="1103" t="n"/>
-      <c r="S188" s="1106" t="n"/>
+      <c r="S188" s="1105" t="n"/>
       <c r="T188" s="1097" t="n"/>
       <c r="U188" s="988" t="n"/>
       <c r="V188" s="988" t="n"/>
@@ -50076,7 +50222,7 @@
       <c r="P189" s="1102" t="n"/>
       <c r="Q189" s="1102" t="n"/>
       <c r="R189" s="1103" t="n"/>
-      <c r="S189" s="1106" t="n"/>
+      <c r="S189" s="1105" t="n"/>
       <c r="T189" s="1097" t="n"/>
       <c r="U189" s="988" t="n"/>
       <c r="V189" s="988" t="n"/>
@@ -50102,7 +50248,7 @@
       <c r="P190" s="1102" t="n"/>
       <c r="Q190" s="1102" t="n"/>
       <c r="R190" s="1103" t="n"/>
-      <c r="S190" s="1106" t="n"/>
+      <c r="S190" s="1105" t="n"/>
       <c r="T190" s="1097" t="n"/>
       <c r="U190" s="988" t="n"/>
       <c r="V190" s="988" t="n"/>
@@ -50128,7 +50274,7 @@
       <c r="P191" s="1102" t="n"/>
       <c r="Q191" s="1102" t="n"/>
       <c r="R191" s="1103" t="n"/>
-      <c r="S191" s="1106" t="n"/>
+      <c r="S191" s="1105" t="n"/>
       <c r="T191" s="1097" t="n"/>
       <c r="U191" s="988" t="n"/>
       <c r="V191" s="988" t="n"/>
@@ -50154,7 +50300,7 @@
       <c r="P192" s="1102" t="n"/>
       <c r="Q192" s="1102" t="n"/>
       <c r="R192" s="1103" t="n"/>
-      <c r="S192" s="1106" t="n"/>
+      <c r="S192" s="1105" t="n"/>
       <c r="T192" s="1097" t="n"/>
       <c r="U192" s="988" t="n"/>
       <c r="V192" s="988" t="n"/>
@@ -50180,7 +50326,7 @@
       <c r="P193" s="1102" t="n"/>
       <c r="Q193" s="1102" t="n"/>
       <c r="R193" s="1103" t="n"/>
-      <c r="S193" s="1106" t="n"/>
+      <c r="S193" s="1105" t="n"/>
       <c r="T193" s="1097" t="n"/>
       <c r="U193" s="988" t="n"/>
       <c r="V193" s="988" t="n"/>
@@ -50206,7 +50352,7 @@
       <c r="P194" s="1102" t="n"/>
       <c r="Q194" s="1102" t="n"/>
       <c r="R194" s="1103" t="n"/>
-      <c r="S194" s="1106" t="n"/>
+      <c r="S194" s="1105" t="n"/>
       <c r="T194" s="1097" t="n"/>
       <c r="U194" s="988" t="n"/>
       <c r="V194" s="988" t="n"/>
@@ -50232,7 +50378,7 @@
       <c r="P195" s="1102" t="n"/>
       <c r="Q195" s="1102" t="n"/>
       <c r="R195" s="1103" t="n"/>
-      <c r="S195" s="1106" t="n"/>
+      <c r="S195" s="1105" t="n"/>
       <c r="T195" s="1097" t="n"/>
       <c r="U195" s="988" t="n"/>
       <c r="V195" s="988" t="n"/>
@@ -50258,7 +50404,7 @@
       <c r="P196" s="1102" t="n"/>
       <c r="Q196" s="1102" t="n"/>
       <c r="R196" s="1103" t="n"/>
-      <c r="S196" s="1106" t="n"/>
+      <c r="S196" s="1105" t="n"/>
       <c r="T196" s="1097" t="n"/>
       <c r="U196" s="988" t="n"/>
       <c r="V196" s="988" t="n"/>
@@ -50284,7 +50430,7 @@
       <c r="P197" s="1102" t="n"/>
       <c r="Q197" s="1102" t="n"/>
       <c r="R197" s="1103" t="n"/>
-      <c r="S197" s="1106" t="n"/>
+      <c r="S197" s="1105" t="n"/>
       <c r="T197" s="1097" t="n"/>
       <c r="U197" s="988" t="n"/>
       <c r="V197" s="988" t="n"/>
@@ -50310,7 +50456,7 @@
       <c r="P198" s="1102" t="n"/>
       <c r="Q198" s="1102" t="n"/>
       <c r="R198" s="1103" t="n"/>
-      <c r="S198" s="1106" t="n"/>
+      <c r="S198" s="1105" t="n"/>
       <c r="T198" s="1097" t="n"/>
       <c r="U198" s="988" t="n"/>
       <c r="V198" s="988" t="n"/>
@@ -50336,7 +50482,7 @@
       <c r="P199" s="1102" t="n"/>
       <c r="Q199" s="1102" t="n"/>
       <c r="R199" s="1103" t="n"/>
-      <c r="S199" s="1106" t="n"/>
+      <c r="S199" s="1105" t="n"/>
       <c r="T199" s="1097" t="n"/>
       <c r="U199" s="988" t="n"/>
       <c r="V199" s="988" t="n"/>
@@ -50362,7 +50508,7 @@
       <c r="P200" s="1102" t="n"/>
       <c r="Q200" s="1102" t="n"/>
       <c r="R200" s="1103" t="n"/>
-      <c r="S200" s="1106" t="n"/>
+      <c r="S200" s="1105" t="n"/>
       <c r="T200" s="1097" t="n"/>
       <c r="U200" s="988" t="n"/>
       <c r="V200" s="988" t="n"/>
@@ -50388,7 +50534,7 @@
       <c r="P201" s="1102" t="n"/>
       <c r="Q201" s="1102" t="n"/>
       <c r="R201" s="1103" t="n"/>
-      <c r="S201" s="1106" t="n"/>
+      <c r="S201" s="1105" t="n"/>
       <c r="T201" s="1097" t="n"/>
       <c r="U201" s="988" t="n"/>
       <c r="V201" s="988" t="n"/>
@@ -50414,7 +50560,7 @@
       <c r="P202" s="1102" t="n"/>
       <c r="Q202" s="1102" t="n"/>
       <c r="R202" s="1103" t="n"/>
-      <c r="S202" s="1106" t="n"/>
+      <c r="S202" s="1105" t="n"/>
       <c r="T202" s="1097" t="n"/>
       <c r="U202" s="988" t="n"/>
       <c r="V202" s="988" t="n"/>
@@ -50440,7 +50586,7 @@
       <c r="P203" s="1102" t="n"/>
       <c r="Q203" s="1102" t="n"/>
       <c r="R203" s="1103" t="n"/>
-      <c r="S203" s="1106" t="n"/>
+      <c r="S203" s="1105" t="n"/>
       <c r="T203" s="1097" t="n"/>
       <c r="U203" s="988" t="n"/>
       <c r="V203" s="988" t="n"/>
@@ -50466,7 +50612,7 @@
       <c r="P204" s="1102" t="n"/>
       <c r="Q204" s="1102" t="n"/>
       <c r="R204" s="1103" t="n"/>
-      <c r="S204" s="1106" t="n"/>
+      <c r="S204" s="1105" t="n"/>
       <c r="T204" s="1097" t="n"/>
       <c r="U204" s="988" t="n"/>
       <c r="V204" s="988" t="n"/>
@@ -50492,7 +50638,7 @@
       <c r="P205" s="1102" t="n"/>
       <c r="Q205" s="1102" t="n"/>
       <c r="R205" s="1103" t="n"/>
-      <c r="S205" s="1106" t="n"/>
+      <c r="S205" s="1105" t="n"/>
       <c r="T205" s="1097" t="n"/>
       <c r="U205" s="988" t="n"/>
       <c r="V205" s="988" t="n"/>
@@ -50518,7 +50664,7 @@
       <c r="P206" s="1102" t="n"/>
       <c r="Q206" s="1102" t="n"/>
       <c r="R206" s="1103" t="n"/>
-      <c r="S206" s="1106" t="n"/>
+      <c r="S206" s="1105" t="n"/>
       <c r="T206" s="1097" t="n"/>
       <c r="U206" s="988" t="n"/>
       <c r="V206" s="988" t="n"/>
@@ -50544,7 +50690,7 @@
       <c r="P207" s="1102" t="n"/>
       <c r="Q207" s="1102" t="n"/>
       <c r="R207" s="1103" t="n"/>
-      <c r="S207" s="1106" t="n"/>
+      <c r="S207" s="1105" t="n"/>
       <c r="T207" s="1097" t="n"/>
       <c r="U207" s="988" t="n"/>
       <c r="V207" s="988" t="n"/>
@@ -50570,7 +50716,7 @@
       <c r="P208" s="1102" t="n"/>
       <c r="Q208" s="1102" t="n"/>
       <c r="R208" s="1103" t="n"/>
-      <c r="S208" s="1106" t="n"/>
+      <c r="S208" s="1105" t="n"/>
       <c r="T208" s="1097" t="n"/>
       <c r="U208" s="988" t="n"/>
       <c r="V208" s="988" t="n"/>
@@ -50596,7 +50742,7 @@
       <c r="P209" s="1102" t="n"/>
       <c r="Q209" s="1102" t="n"/>
       <c r="R209" s="1103" t="n"/>
-      <c r="S209" s="1106" t="n"/>
+      <c r="S209" s="1105" t="n"/>
       <c r="T209" s="1097" t="n"/>
       <c r="U209" s="988" t="n"/>
       <c r="V209" s="988" t="n"/>
@@ -50622,7 +50768,7 @@
       <c r="P210" s="1102" t="n"/>
       <c r="Q210" s="1102" t="n"/>
       <c r="R210" s="1103" t="n"/>
-      <c r="S210" s="1106" t="n"/>
+      <c r="S210" s="1105" t="n"/>
       <c r="T210" s="1097" t="n"/>
       <c r="U210" s="988" t="n"/>
       <c r="V210" s="988" t="n"/>
@@ -50648,7 +50794,7 @@
       <c r="P211" s="1102" t="n"/>
       <c r="Q211" s="1102" t="n"/>
       <c r="R211" s="1103" t="n"/>
-      <c r="S211" s="1106" t="n"/>
+      <c r="S211" s="1105" t="n"/>
       <c r="T211" s="1097" t="n"/>
       <c r="U211" s="988" t="n"/>
       <c r="V211" s="988" t="n"/>
@@ -50674,7 +50820,7 @@
       <c r="P212" s="1102" t="n"/>
       <c r="Q212" s="1102" t="n"/>
       <c r="R212" s="1103" t="n"/>
-      <c r="S212" s="1106" t="n"/>
+      <c r="S212" s="1105" t="n"/>
       <c r="T212" s="1097" t="n"/>
       <c r="U212" s="988" t="n"/>
       <c r="V212" s="988" t="n"/>
@@ -50700,7 +50846,7 @@
       <c r="P213" s="1102" t="n"/>
       <c r="Q213" s="1102" t="n"/>
       <c r="R213" s="1103" t="n"/>
-      <c r="S213" s="1106" t="n"/>
+      <c r="S213" s="1105" t="n"/>
       <c r="T213" s="1097" t="n"/>
       <c r="U213" s="988" t="n"/>
       <c r="V213" s="988" t="n"/>
@@ -50726,7 +50872,7 @@
       <c r="P214" s="1102" t="n"/>
       <c r="Q214" s="1102" t="n"/>
       <c r="R214" s="1103" t="n"/>
-      <c r="S214" s="1106" t="n"/>
+      <c r="S214" s="1105" t="n"/>
       <c r="T214" s="1097" t="n"/>
       <c r="U214" s="988" t="n"/>
       <c r="V214" s="988" t="n"/>
@@ -50752,7 +50898,7 @@
       <c r="P215" s="1102" t="n"/>
       <c r="Q215" s="1102" t="n"/>
       <c r="R215" s="1103" t="n"/>
-      <c r="S215" s="1106" t="n"/>
+      <c r="S215" s="1105" t="n"/>
       <c r="T215" s="1097" t="n"/>
       <c r="U215" s="988" t="n"/>
       <c r="V215" s="988" t="n"/>
@@ -50778,7 +50924,7 @@
       <c r="P216" s="1102" t="n"/>
       <c r="Q216" s="1102" t="n"/>
       <c r="R216" s="1103" t="n"/>
-      <c r="S216" s="1106" t="n"/>
+      <c r="S216" s="1105" t="n"/>
       <c r="T216" s="1097" t="n"/>
       <c r="U216" s="988" t="n"/>
       <c r="V216" s="988" t="n"/>
@@ -50804,7 +50950,7 @@
       <c r="P217" s="1102" t="n"/>
       <c r="Q217" s="1102" t="n"/>
       <c r="R217" s="1103" t="n"/>
-      <c r="S217" s="1106" t="n"/>
+      <c r="S217" s="1105" t="n"/>
       <c r="T217" s="1097" t="n"/>
       <c r="U217" s="988" t="n"/>
       <c r="V217" s="988" t="n"/>
@@ -50830,7 +50976,7 @@
       <c r="P218" s="1102" t="n"/>
       <c r="Q218" s="1102" t="n"/>
       <c r="R218" s="1103" t="n"/>
-      <c r="S218" s="1106" t="n"/>
+      <c r="S218" s="1105" t="n"/>
       <c r="T218" s="1097" t="n"/>
       <c r="U218" s="988" t="n"/>
       <c r="V218" s="988" t="n"/>
@@ -50856,7 +51002,7 @@
       <c r="P219" s="1102" t="n"/>
       <c r="Q219" s="1102" t="n"/>
       <c r="R219" s="1103" t="n"/>
-      <c r="S219" s="1106" t="n"/>
+      <c r="S219" s="1105" t="n"/>
       <c r="T219" s="1097" t="n"/>
       <c r="U219" s="988" t="n"/>
       <c r="V219" s="988" t="n"/>
@@ -50882,7 +51028,7 @@
       <c r="P220" s="1102" t="n"/>
       <c r="Q220" s="1102" t="n"/>
       <c r="R220" s="1103" t="n"/>
-      <c r="S220" s="1106" t="n"/>
+      <c r="S220" s="1105" t="n"/>
       <c r="T220" s="1097" t="n"/>
       <c r="U220" s="988" t="n"/>
       <c r="V220" s="988" t="n"/>
@@ -50908,7 +51054,7 @@
       <c r="P221" s="1102" t="n"/>
       <c r="Q221" s="1102" t="n"/>
       <c r="R221" s="1103" t="n"/>
-      <c r="S221" s="1106" t="n"/>
+      <c r="S221" s="1105" t="n"/>
       <c r="T221" s="1097" t="n"/>
       <c r="U221" s="988" t="n"/>
       <c r="V221" s="988" t="n"/>
@@ -50934,7 +51080,7 @@
       <c r="P222" s="1102" t="n"/>
       <c r="Q222" s="1102" t="n"/>
       <c r="R222" s="1103" t="n"/>
-      <c r="S222" s="1106" t="n"/>
+      <c r="S222" s="1105" t="n"/>
       <c r="T222" s="1097" t="n"/>
       <c r="U222" s="988" t="n"/>
       <c r="V222" s="988" t="n"/>
@@ -50960,7 +51106,7 @@
       <c r="P223" s="1102" t="n"/>
       <c r="Q223" s="1102" t="n"/>
       <c r="R223" s="1103" t="n"/>
-      <c r="S223" s="1106" t="n"/>
+      <c r="S223" s="1105" t="n"/>
       <c r="T223" s="1097" t="n"/>
       <c r="U223" s="988" t="n"/>
       <c r="V223" s="988" t="n"/>
@@ -50986,7 +51132,7 @@
       <c r="P224" s="1102" t="n"/>
       <c r="Q224" s="1102" t="n"/>
       <c r="R224" s="1103" t="n"/>
-      <c r="S224" s="1106" t="n"/>
+      <c r="S224" s="1105" t="n"/>
       <c r="T224" s="1097" t="n"/>
       <c r="U224" s="988" t="n"/>
       <c r="V224" s="988" t="n"/>
@@ -51012,7 +51158,7 @@
       <c r="P225" s="1102" t="n"/>
       <c r="Q225" s="1102" t="n"/>
       <c r="R225" s="1103" t="n"/>
-      <c r="S225" s="1106" t="n"/>
+      <c r="S225" s="1105" t="n"/>
       <c r="T225" s="1097" t="n"/>
       <c r="U225" s="988" t="n"/>
       <c r="V225" s="988" t="n"/>
@@ -51038,7 +51184,7 @@
       <c r="P226" s="1102" t="n"/>
       <c r="Q226" s="1102" t="n"/>
       <c r="R226" s="1103" t="n"/>
-      <c r="S226" s="1106" t="n"/>
+      <c r="S226" s="1105" t="n"/>
       <c r="T226" s="1097" t="n"/>
       <c r="U226" s="988" t="n"/>
       <c r="V226" s="988" t="n"/>
@@ -51064,7 +51210,7 @@
       <c r="P227" s="1102" t="n"/>
       <c r="Q227" s="1102" t="n"/>
       <c r="R227" s="1103" t="n"/>
-      <c r="S227" s="1106" t="n"/>
+      <c r="S227" s="1105" t="n"/>
       <c r="T227" s="1097" t="n"/>
       <c r="U227" s="988" t="n"/>
       <c r="V227" s="988" t="n"/>
@@ -51090,7 +51236,7 @@
       <c r="P228" s="1102" t="n"/>
       <c r="Q228" s="1102" t="n"/>
       <c r="R228" s="1103" t="n"/>
-      <c r="S228" s="1106" t="n"/>
+      <c r="S228" s="1105" t="n"/>
       <c r="T228" s="1097" t="n"/>
       <c r="U228" s="988" t="n"/>
       <c r="V228" s="988" t="n"/>
@@ -51116,7 +51262,7 @@
       <c r="P229" s="1102" t="n"/>
       <c r="Q229" s="1102" t="n"/>
       <c r="R229" s="1103" t="n"/>
-      <c r="S229" s="1106" t="n"/>
+      <c r="S229" s="1105" t="n"/>
       <c r="T229" s="1097" t="n"/>
       <c r="U229" s="988" t="n"/>
       <c r="V229" s="988" t="n"/>
@@ -51142,7 +51288,7 @@
       <c r="P230" s="1102" t="n"/>
       <c r="Q230" s="1102" t="n"/>
       <c r="R230" s="1103" t="n"/>
-      <c r="S230" s="1106" t="n"/>
+      <c r="S230" s="1105" t="n"/>
       <c r="T230" s="1097" t="n"/>
       <c r="U230" s="988" t="n"/>
       <c r="V230" s="988" t="n"/>
@@ -51168,7 +51314,7 @@
       <c r="P231" s="1102" t="n"/>
       <c r="Q231" s="1102" t="n"/>
       <c r="R231" s="1103" t="n"/>
-      <c r="S231" s="1106" t="n"/>
+      <c r="S231" s="1105" t="n"/>
       <c r="T231" s="1097" t="n"/>
       <c r="U231" s="988" t="n"/>
       <c r="V231" s="988" t="n"/>
@@ -51194,7 +51340,7 @@
       <c r="P232" s="1102" t="n"/>
       <c r="Q232" s="1102" t="n"/>
       <c r="R232" s="1103" t="n"/>
-      <c r="S232" s="1106" t="n"/>
+      <c r="S232" s="1105" t="n"/>
       <c r="T232" s="1097" t="n"/>
       <c r="U232" s="988" t="n"/>
       <c r="V232" s="988" t="n"/>
@@ -51220,7 +51366,7 @@
       <c r="P233" s="1102" t="n"/>
       <c r="Q233" s="1102" t="n"/>
       <c r="R233" s="1103" t="n"/>
-      <c r="S233" s="1106" t="n"/>
+      <c r="S233" s="1105" t="n"/>
       <c r="T233" s="1097" t="n"/>
       <c r="U233" s="988" t="n"/>
       <c r="V233" s="988" t="n"/>
@@ -51246,7 +51392,7 @@
       <c r="P234" s="1102" t="n"/>
       <c r="Q234" s="1102" t="n"/>
       <c r="R234" s="1103" t="n"/>
-      <c r="S234" s="1106" t="n"/>
+      <c r="S234" s="1105" t="n"/>
       <c r="T234" s="1097" t="n"/>
       <c r="U234" s="988" t="n"/>
       <c r="V234" s="988" t="n"/>
@@ -51272,7 +51418,7 @@
       <c r="P235" s="1102" t="n"/>
       <c r="Q235" s="1102" t="n"/>
       <c r="R235" s="1103" t="n"/>
-      <c r="S235" s="1106" t="n"/>
+      <c r="S235" s="1105" t="n"/>
       <c r="T235" s="1097" t="n"/>
       <c r="U235" s="988" t="n"/>
       <c r="V235" s="988" t="n"/>
@@ -51298,7 +51444,7 @@
       <c r="P236" s="1102" t="n"/>
       <c r="Q236" s="1102" t="n"/>
       <c r="R236" s="1103" t="n"/>
-      <c r="S236" s="1106" t="n"/>
+      <c r="S236" s="1105" t="n"/>
       <c r="T236" s="1097" t="n"/>
       <c r="U236" s="988" t="n"/>
       <c r="V236" s="988" t="n"/>
@@ -51324,7 +51470,7 @@
       <c r="P237" s="1102" t="n"/>
       <c r="Q237" s="1102" t="n"/>
       <c r="R237" s="1103" t="n"/>
-      <c r="S237" s="1106" t="n"/>
+      <c r="S237" s="1105" t="n"/>
       <c r="T237" s="1097" t="n"/>
       <c r="U237" s="988" t="n"/>
       <c r="V237" s="988" t="n"/>
@@ -51350,7 +51496,7 @@
       <c r="P238" s="1102" t="n"/>
       <c r="Q238" s="1102" t="n"/>
       <c r="R238" s="1103" t="n"/>
-      <c r="S238" s="1106" t="n"/>
+      <c r="S238" s="1105" t="n"/>
       <c r="T238" s="1097" t="n"/>
       <c r="U238" s="988" t="n"/>
       <c r="V238" s="988" t="n"/>
@@ -51376,7 +51522,7 @@
       <c r="P239" s="1102" t="n"/>
       <c r="Q239" s="1102" t="n"/>
       <c r="R239" s="1103" t="n"/>
-      <c r="S239" s="1106" t="n"/>
+      <c r="S239" s="1105" t="n"/>
       <c r="T239" s="1097" t="n"/>
       <c r="U239" s="988" t="n"/>
       <c r="V239" s="988" t="n"/>
@@ -51402,7 +51548,7 @@
       <c r="P240" s="1102" t="n"/>
       <c r="Q240" s="1102" t="n"/>
       <c r="R240" s="1103" t="n"/>
-      <c r="S240" s="1106" t="n"/>
+      <c r="S240" s="1105" t="n"/>
       <c r="T240" s="1097" t="n"/>
       <c r="U240" s="988" t="n"/>
       <c r="V240" s="988" t="n"/>
@@ -51428,7 +51574,7 @@
       <c r="P241" s="1102" t="n"/>
       <c r="Q241" s="1102" t="n"/>
       <c r="R241" s="1103" t="n"/>
-      <c r="S241" s="1106" t="n"/>
+      <c r="S241" s="1105" t="n"/>
       <c r="T241" s="1097" t="n"/>
       <c r="U241" s="988" t="n"/>
       <c r="V241" s="988" t="n"/>
@@ -51454,7 +51600,7 @@
       <c r="P242" s="1102" t="n"/>
       <c r="Q242" s="1102" t="n"/>
       <c r="R242" s="1103" t="n"/>
-      <c r="S242" s="1106" t="n"/>
+      <c r="S242" s="1105" t="n"/>
       <c r="T242" s="1097" t="n"/>
       <c r="U242" s="988" t="n"/>
       <c r="V242" s="988" t="n"/>
@@ -51480,7 +51626,7 @@
       <c r="P243" s="1102" t="n"/>
       <c r="Q243" s="1102" t="n"/>
       <c r="R243" s="1103" t="n"/>
-      <c r="S243" s="1106" t="n"/>
+      <c r="S243" s="1105" t="n"/>
       <c r="T243" s="1097" t="n"/>
       <c r="U243" s="988" t="n"/>
       <c r="V243" s="988" t="n"/>
@@ -51506,7 +51652,7 @@
       <c r="P244" s="1102" t="n"/>
       <c r="Q244" s="1102" t="n"/>
       <c r="R244" s="1103" t="n"/>
-      <c r="S244" s="1106" t="n"/>
+      <c r="S244" s="1105" t="n"/>
       <c r="T244" s="1097" t="n"/>
       <c r="U244" s="988" t="n"/>
       <c r="V244" s="988" t="n"/>
@@ -51532,7 +51678,7 @@
       <c r="P245" s="1102" t="n"/>
       <c r="Q245" s="1102" t="n"/>
       <c r="R245" s="1103" t="n"/>
-      <c r="S245" s="1106" t="n"/>
+      <c r="S245" s="1105" t="n"/>
       <c r="T245" s="1097" t="n"/>
       <c r="U245" s="988" t="n"/>
       <c r="V245" s="988" t="n"/>
@@ -51558,7 +51704,7 @@
       <c r="P246" s="1102" t="n"/>
       <c r="Q246" s="1102" t="n"/>
       <c r="R246" s="1103" t="n"/>
-      <c r="S246" s="1106" t="n"/>
+      <c r="S246" s="1105" t="n"/>
       <c r="T246" s="1097" t="n"/>
       <c r="U246" s="988" t="n"/>
       <c r="V246" s="988" t="n"/>
@@ -51584,7 +51730,7 @@
       <c r="P247" s="1102" t="n"/>
       <c r="Q247" s="1102" t="n"/>
       <c r="R247" s="1103" t="n"/>
-      <c r="S247" s="1106" t="n"/>
+      <c r="S247" s="1105" t="n"/>
       <c r="T247" s="1097" t="n"/>
       <c r="U247" s="988" t="n"/>
       <c r="V247" s="988" t="n"/>
@@ -51610,7 +51756,7 @@
       <c r="P248" s="1102" t="n"/>
       <c r="Q248" s="1102" t="n"/>
       <c r="R248" s="1103" t="n"/>
-      <c r="S248" s="1106" t="n"/>
+      <c r="S248" s="1105" t="n"/>
       <c r="T248" s="1097" t="n"/>
       <c r="U248" s="988" t="n"/>
       <c r="V248" s="988" t="n"/>
@@ -51636,7 +51782,7 @@
       <c r="P249" s="1102" t="n"/>
       <c r="Q249" s="1102" t="n"/>
       <c r="R249" s="1103" t="n"/>
-      <c r="S249" s="1106" t="n"/>
+      <c r="S249" s="1105" t="n"/>
       <c r="T249" s="1097" t="n"/>
       <c r="U249" s="988" t="n"/>
       <c r="V249" s="988" t="n"/>
@@ -51662,7 +51808,7 @@
       <c r="P250" s="1102" t="n"/>
       <c r="Q250" s="1102" t="n"/>
       <c r="R250" s="1103" t="n"/>
-      <c r="S250" s="1106" t="n"/>
+      <c r="S250" s="1105" t="n"/>
       <c r="T250" s="1097" t="n"/>
       <c r="U250" s="988" t="n"/>
       <c r="V250" s="988" t="n"/>
@@ -51688,7 +51834,7 @@
       <c r="P251" s="1102" t="n"/>
       <c r="Q251" s="1102" t="n"/>
       <c r="R251" s="1103" t="n"/>
-      <c r="S251" s="1106" t="n"/>
+      <c r="S251" s="1105" t="n"/>
       <c r="T251" s="1097" t="n"/>
       <c r="U251" s="988" t="n"/>
       <c r="V251" s="988" t="n"/>
@@ -51714,7 +51860,7 @@
       <c r="P252" s="1102" t="n"/>
       <c r="Q252" s="1102" t="n"/>
       <c r="R252" s="1103" t="n"/>
-      <c r="S252" s="1106" t="n"/>
+      <c r="S252" s="1105" t="n"/>
       <c r="T252" s="1097" t="n"/>
       <c r="U252" s="988" t="n"/>
       <c r="V252" s="988" t="n"/>
@@ -51740,7 +51886,7 @@
       <c r="P253" s="1102" t="n"/>
       <c r="Q253" s="1102" t="n"/>
       <c r="R253" s="1103" t="n"/>
-      <c r="S253" s="1106" t="n"/>
+      <c r="S253" s="1105" t="n"/>
       <c r="T253" s="1097" t="n"/>
       <c r="U253" s="988" t="n"/>
       <c r="V253" s="988" t="n"/>
@@ -51766,7 +51912,7 @@
       <c r="P254" s="1102" t="n"/>
       <c r="Q254" s="1102" t="n"/>
       <c r="R254" s="1103" t="n"/>
-      <c r="S254" s="1106" t="n"/>
+      <c r="S254" s="1105" t="n"/>
       <c r="T254" s="1097" t="n"/>
       <c r="U254" s="988" t="n"/>
       <c r="V254" s="988" t="n"/>
@@ -51792,7 +51938,7 @@
       <c r="P255" s="1102" t="n"/>
       <c r="Q255" s="1102" t="n"/>
       <c r="R255" s="1103" t="n"/>
-      <c r="S255" s="1106" t="n"/>
+      <c r="S255" s="1105" t="n"/>
       <c r="T255" s="1097" t="n"/>
       <c r="U255" s="988" t="n"/>
       <c r="V255" s="988" t="n"/>
@@ -51818,7 +51964,7 @@
       <c r="P256" s="1102" t="n"/>
       <c r="Q256" s="1102" t="n"/>
       <c r="R256" s="1103" t="n"/>
-      <c r="S256" s="1106" t="n"/>
+      <c r="S256" s="1105" t="n"/>
       <c r="T256" s="1097" t="n"/>
       <c r="U256" s="988" t="n"/>
       <c r="V256" s="988" t="n"/>
@@ -51844,7 +51990,7 @@
       <c r="P257" s="1102" t="n"/>
       <c r="Q257" s="1102" t="n"/>
       <c r="R257" s="1103" t="n"/>
-      <c r="S257" s="1106" t="n"/>
+      <c r="S257" s="1105" t="n"/>
       <c r="T257" s="1097" t="n"/>
       <c r="U257" s="988" t="n"/>
       <c r="V257" s="988" t="n"/>
@@ -51870,7 +52016,7 @@
       <c r="P258" s="1102" t="n"/>
       <c r="Q258" s="1102" t="n"/>
       <c r="R258" s="1103" t="n"/>
-      <c r="S258" s="1106" t="n"/>
+      <c r="S258" s="1105" t="n"/>
       <c r="T258" s="1097" t="n"/>
       <c r="U258" s="988" t="n"/>
       <c r="V258" s="988" t="n"/>
@@ -51896,7 +52042,7 @@
       <c r="P259" s="1102" t="n"/>
       <c r="Q259" s="1102" t="n"/>
       <c r="R259" s="1103" t="n"/>
-      <c r="S259" s="1106" t="n"/>
+      <c r="S259" s="1105" t="n"/>
       <c r="T259" s="1097" t="n"/>
       <c r="U259" s="988" t="n"/>
       <c r="V259" s="988" t="n"/>

</xml_diff>